<commit_message>
Add JWT token lifetime setting and update QA testing guide with environment reset instructions
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -10,7 +10,7 @@
     <sheet name="QA Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'QA Test Cases'!$A$1:$I$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'QA Test Cases'!$A$1:$I$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -52,8 +52,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E2F3"/>
-        <bgColor rgb="00D9E2F3"/>
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,7 +106,7 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -479,18 +479,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,27 +516,27 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Steps to reproduce</t>
+          <t>Steps</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Expected result</t>
+          <t>Expected</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Actual result</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Test data (if any)</t>
+          <t>Test data</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Additional comments (if any)</t>
+          <t>Comments</t>
         </is>
       </c>
     </row>
@@ -558,12 +558,12 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-001</t>
+          <t>TC-101</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Valid login returns token</t>
+          <t>Valid login</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -574,28 +574,31 @@
       <c r="D3" s="5" t="inlineStr"/>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with valid OS username/password
-2. Inspect response body</t>
+          <t>POST /auth/token with valid OS username/password</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>200, response contains 'access_token' and 'token_type: "bearer"'</t>
+          <t>200; response contains access_token and token_type: "bearer"</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Username: qa-admin, Password: QaPass-admin!</t>
+        </is>
+      </c>
       <c r="I3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-002</t>
+          <t>TC-102</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Invalid password returns 401</t>
+          <t>Invalid password</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -606,27 +609,31 @@
       <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with valid username but wrong password</t>
+          <t>POST /auth/token with wrong password</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>401, 'Invalid credentials'</t>
+          <t>401, Invalid credentials</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Username: qa-admin, Password: wrong</t>
+        </is>
+      </c>
       <c r="I4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-003</t>
+          <t>TC-103</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Unknown user returns 401</t>
+          <t>Unknown user</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -637,27 +644,31 @@
       <c r="D5" s="5" t="inlineStr"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with non-existent username</t>
+          <t>POST /auth/token with non-existent username</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>401, 'Invalid credentials'</t>
+          <t>401, Invalid credentials</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Username: nonexistent</t>
+        </is>
+      </c>
       <c r="I5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-004</t>
+          <t>TC-104</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Missing username returns 422</t>
+          <t>Missing username</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -668,7 +679,7 @@
       <c r="D6" s="5" t="inlineStr"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with body: {"password": "x"}</t>
+          <t>POST /auth/token with {"password": "x"}</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -683,12 +694,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-005</t>
+          <t>TC-105</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Missing password returns 422</t>
+          <t>Missing password</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -699,7 +710,7 @@
       <c r="D7" s="5" t="inlineStr"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with body: {"username": "x"}</t>
+          <t>POST /auth/token with {"username": "x"}</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -714,12 +725,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-006</t>
+          <t>TC-106</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Empty username returns 422</t>
+          <t>Empty username</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -730,7 +741,7 @@
       <c r="D8" s="5" t="inlineStr"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with body: {"username": "", "password": "x"}</t>
+          <t>POST /auth/token with {"username": "", "password": "x"}</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -745,7 +756,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-007</t>
+          <t>TC-107</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -761,14 +772,12 @@
       <c r="D9" s="5" t="inlineStr"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with valid credentials
-2. Decode the JWT from the response
-3. Inspect the 'roles' claim</t>
+          <t>Decode JWT from login response</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>'roles' matches group mapping in LOCAL_GROUP_ROLE_MAP</t>
+          <t>roles matches group mapping in LOCAL_GROUP_ROLE_MAP</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr"/>
@@ -778,7 +787,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-008</t>
+          <t>TC-108</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -794,14 +803,12 @@
       <c r="D10" s="5" t="inlineStr"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with valid credentials
-2. Decode the JWT from the response
-3. Inspect the 'groups' claim</t>
+          <t>Decode JWT from login response</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>'groups' lists the user's OS groups</t>
+          <t>groups lists the user's OS groups</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr"/>
@@ -811,12 +818,12 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-009</t>
+          <t>TC-109</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Token is usable for API calls</t>
+          <t>Token is usable</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -827,13 +834,12 @@
       <c r="D11" s="5" t="inlineStr"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with valid credentials
-2. Use returned token to call GET /drives</t>
+          <t>Use returned token to call GET /drives</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>200 response from /drives</t>
+          <t>200</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
@@ -843,12 +849,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-010</t>
+          <t>TC-110</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Login success audit log</t>
+          <t>Login audit log</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -859,8 +865,7 @@
       <c r="D12" s="5" t="inlineStr"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with valid credentials
-2. GET /audit?action=AUTH_SUCCESS</t>
+          <t>GET /audit?action=AUTH_SUCCESS after successful login</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -875,12 +880,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-011</t>
+          <t>TC-111</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Login failure audit log</t>
+          <t>Failed login audit log</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -891,8 +896,7 @@
       <c r="D13" s="5" t="inlineStr"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token with invalid credentials
-2. GET /audit?action=AUTH_FAILURE</t>
+          <t>GET /audit?action=AUTH_FAILURE after failed login</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -907,12 +911,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>LOGIN-012</t>
+          <t>TC-112</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Login requires no auth header</t>
+          <t>No auth required for login</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -923,8 +927,7 @@
       <c r="D14" s="5" t="inlineStr"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>1. POST /auth/token without Authorization header
-2. Provide valid username/password</t>
+          <t>POST /auth/token without Authorization header</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -954,12 +957,12 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>AUTH-001</t>
+          <t>TC-201</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>No token returns 401</t>
+          <t>No token</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -970,7 +973,7 @@
       <c r="D16" s="5" t="inlineStr"/>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>1. GET /drives without Authorization header</t>
+          <t>curl -sk https://localhost:8443/drives (no auth header)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -985,12 +988,12 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>AUTH-002</t>
+          <t>TC-202</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Garbage token returns 401</t>
+          <t>Garbage token</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1001,7 +1004,7 @@
       <c r="D17" s="5" t="inlineStr"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>1. GET /drives with header: Authorization: Bearer not.a.real.token</t>
+          <t>Authorization: Bearer not.a.real.token</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1016,12 +1019,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>AUTH-003</t>
+          <t>TC-203</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Expired token returns 401</t>
+          <t>Expired token</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1032,8 +1035,7 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>1. Generate token with exp in the past
-2. Use token to call any endpoint</t>
+          <t>Generate token with exp = time.time() - 60</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1048,12 +1050,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>AUTH-004</t>
+          <t>TC-204</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Processor cannot add mount</t>
+          <t>Processor adds mount</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1064,7 +1066,7 @@
       <c r="D19" s="5" t="inlineStr"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>1. POST /mounts with processor-role token</t>
+          <t>POST /mounts with processor token</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -1073,18 +1075,22 @@
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr"/>
-      <c r="H19" s="5" t="inlineStr"/>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Login as qa-processor</t>
+        </is>
+      </c>
       <c r="I19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>AUTH-005</t>
+          <t>TC-205</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Processor cannot initialize drive</t>
+          <t>Processor initializes drive</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -1095,7 +1101,7 @@
       <c r="D20" s="5" t="inlineStr"/>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>1. POST /drives/{id}/initialize with processor-role token</t>
+          <t>POST /drives/{id}/initialize with processor token</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1104,18 +1110,22 @@
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Login as qa-processor</t>
+        </is>
+      </c>
       <c r="I20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>AUTH-006</t>
+          <t>TC-206</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Processor cannot read audit</t>
+          <t>Processor reads audit</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -1126,7 +1136,7 @@
       <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>1. GET /audit with processor-role token</t>
+          <t>GET /audit with processor token</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1135,18 +1145,22 @@
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Login as qa-processor</t>
+        </is>
+      </c>
       <c r="I21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>AUTH-007</t>
+          <t>TC-207</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Auditor can read audit</t>
+          <t>Auditor reads audit</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -1157,7 +1171,7 @@
       <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>1. GET /audit with auditor-role token</t>
+          <t>GET /audit with auditor token</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1166,18 +1180,22 @@
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="5" t="inlineStr"/>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Login as qa-auditor</t>
+        </is>
+      </c>
       <c r="I22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>AUTH-008</t>
+          <t>TC-208</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Processor can create job</t>
+          <t>Processor creates job</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -1188,7 +1206,7 @@
       <c r="D23" s="5" t="inlineStr"/>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>1. POST /jobs with processor-role token</t>
+          <t>POST /jobs with processor token</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1197,18 +1215,22 @@
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Login as qa-processor</t>
+        </is>
+      </c>
       <c r="I23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>AUTH-009</t>
+          <t>TC-209</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Error responses include trace_id</t>
+          <t>Error responses have trace_id</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -1219,13 +1241,12 @@
       <c r="D24" s="5" t="inlineStr"/>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>1. Trigger any 4xx/5xx error
-2. Inspect JSON response body</t>
+          <t>Inspect any 4xx/5xx JSON body</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>trace_id field present in response</t>
+          <t>trace_id field present</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr"/>
@@ -1250,12 +1271,12 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>ISO-001</t>
+          <t>TC-301</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Initialize drive with project</t>
+          <t>Initialize AVAILABLE drive with PROJ-A</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -1266,27 +1287,31 @@
       <c r="D26" s="5" t="inlineStr"/>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>1. Initialize an AVAILABLE drive with project_id: PROJ-A</t>
+          <t>POST /drives/{id}/initialize with project_id: PROJ-A</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>200, drive state → IN_USE</t>
+          <t>200, state → IN_USE</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr"/>
-      <c r="H26" s="5" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Drive must be AVAILABLE</t>
+        </is>
+      </c>
       <c r="I26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>ISO-002</t>
+          <t>TC-302</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Re-initialize with different project rejected</t>
+          <t>Re-initialize with PROJ-B</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -1297,7 +1322,7 @@
       <c r="D27" s="5" t="inlineStr"/>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>1. Initialize same drive with project_id: PROJ-B</t>
+          <t>POST /drives/{id}/initialize with project_id: PROJ-B on same drive</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -1306,18 +1331,22 @@
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr"/>
-      <c r="H27" s="5" t="inlineStr"/>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Same drive as TC-301</t>
+        </is>
+      </c>
       <c r="I27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>ISO-003</t>
+          <t>TC-303</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Isolation violation audit log</t>
+          <t>Audit log for isolation violation</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -1328,8 +1357,7 @@
       <c r="D28" s="5" t="inlineStr"/>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>1. After ISO-002, GET /audit
-2. Search for PROJECT_ISOLATION_VIOLATION</t>
+          <t>GET /audit?action=PROJECT_ISOLATION_VIOLATION</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -1359,7 +1387,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>DRV-001</t>
+          <t>TC-401</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1375,12 +1403,12 @@
       <c r="D30" s="5" t="inlineStr"/>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>1. POST /drives/{id}/initialize on an AVAILABLE drive</t>
+          <t>POST /drives/{id}/initialize on AVAILABLE drive</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>200, drive state → IN_USE</t>
+          <t>200, state → IN_USE</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr"/>
@@ -1390,12 +1418,12 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>DRV-002</t>
+          <t>TC-402</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Initialize an EMPTY drive rejected</t>
+          <t>Initialize an EMPTY drive</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -1406,7 +1434,7 @@
       <c r="D31" s="5" t="inlineStr"/>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>1. POST /drives/{id}/initialize on an EMPTY drive</t>
+          <t>POST /drives/{id}/initialize on EMPTY drive</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -1421,7 +1449,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>DRV-003</t>
+          <t>TC-403</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1437,12 +1465,12 @@
       <c r="D32" s="5" t="inlineStr"/>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>1. POST /drives/{id}/prepare-eject on an IN_USE drive</t>
+          <t>POST /drives/{id}/prepare-eject on IN_USE drive</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>200, drive state → AVAILABLE</t>
+          <t>200, state → AVAILABLE</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr"/>
@@ -1452,12 +1480,12 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>DRV-004</t>
+          <t>TC-404</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Prepare-eject an AVAILABLE drive rejected</t>
+          <t>Prepare-eject an AVAILABLE drive</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -1468,7 +1496,7 @@
       <c r="D33" s="5" t="inlineStr"/>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>1. POST /drives/{id}/prepare-eject on an AVAILABLE drive</t>
+          <t>POST /drives/{id}/prepare-eject on AVAILABLE drive</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -1498,7 +1526,7 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>USB-001</t>
+          <t>TC-501</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -1514,29 +1542,31 @@
       <c r="D35" s="5" t="inlineStr"/>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>1. Plug in a USB drive
-2. Wait 30 seconds
-3. GET /drives</t>
+          <t>Plug in a USB drive, wait 30 seconds, GET /drives</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>New drive appears in EMPTY state</t>
+          <t>New drive in AVAILABLE state (discovery auto-transitions EMPTY → AVAILABLE)</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr"/>
-      <c r="H35" s="5" t="inlineStr"/>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Requires physical USB drive</t>
+        </is>
+      </c>
       <c r="I35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>USB-002</t>
+          <t>TC-502</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>USB topology shows real hardware</t>
+          <t>USB topology</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -1547,7 +1577,7 @@
       <c r="D36" s="5" t="inlineStr"/>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>1. GET /introspection/usb/topology</t>
+          <t>GET /introspection/usb/topology</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -1562,12 +1592,12 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>USB-003</t>
+          <t>TC-503</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Physical eject workflow</t>
+          <t>Physical eject</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -1578,9 +1608,7 @@
       <c r="D37" s="5" t="inlineStr"/>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>1. Initialize drive
-2. POST /drives/{id}/prepare-eject
-3. Physically remove drive</t>
+          <t>Initialize drive → prepare-eject → physically remove</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
@@ -1595,7 +1623,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>USB-004</t>
+          <t>TC-504</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -1611,13 +1639,12 @@
       <c r="D38" s="5" t="inlineStr"/>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>1. Remove a previously initialized drive
-2. Re-insert the same drive</t>
+          <t>Remove and re-insert the same drive</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Drive reappears as EMPTY with same device_identifier</t>
+          <t>Drive reappears as AVAILABLE with same device_identifier (after discovery cycle)</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
@@ -1627,12 +1654,12 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>USB-005</t>
+          <t>TC-505</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Multiple simultaneous drives</t>
+          <t>Multiple drives</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -1643,28 +1670,31 @@
       <c r="D39" s="5" t="inlineStr"/>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>1. Plug in 2+ USB drives simultaneously
-2. GET /drives</t>
+          <t>Plug in 2+ drives simultaneously</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>All drives appear; each can be initialized to different projects</t>
+          <t>All drives appear in /drives; each can be initialized to different projects</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr"/>
-      <c r="H39" s="5" t="inlineStr"/>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Requires 2+ USB drives</t>
+        </is>
+      </c>
       <c r="I39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>USB-006</t>
+          <t>TC-506</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Sync + unmount on eject</t>
+          <t>Sync + unmount</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -1675,15 +1705,12 @@
       <c r="D40" s="5" t="inlineStr"/>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>1. Initialize drive
-2. Create and start a copy job
-3. POST /drives/{id}/prepare-eject
-4. Run 'mount' command on host</t>
+          <t>Initialize drive, create/start a job, then prepare-eject</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Filesystem flushed and unmounted; no partitions from that drive listed in mount output</t>
+          <t>Filesystem flushed and unmounted; mount command shows no partitions from that drive</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr"/>
@@ -1708,12 +1735,12 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>E2E-001</t>
+          <t>TC-601</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Complete data export lifecycle</t>
+          <t>E2E: Set up test data</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -1724,54 +1751,62 @@
       <c r="D42" s="5" t="inlineStr"/>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>1. Create test file share (mkdir /mnt/test-evidence; copy sample files)
-2. POST /mounts to add the mount
-3. Plug in USB drive, wait for auto-discovery
-4. GET /drives — note drive ID
-5. POST /drives/{id}/initialize with project_id: PROJ-E2E
-6. POST /jobs with source_path to test files
-7. POST /jobs/{id}/start
-8. Poll GET /jobs/{id} until status = COMPLETED
-9. POST /jobs/{id}/verify — confirm all files pass
-10. POST /jobs/{id}/manifest
-11. POST /drives/{id}/prepare-eject
-12. Physically remove drive, verify data on another computer
-13. GET /audit — confirm complete chain</t>
+          <t>Create /mnt/test-evidence/case-001 with doc-alpha.txt, doc-bravo.txt, binary-10mb.bin; record sha256sums</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>All steps succeed. Audit trail shows: MOUNT_ADDED → DRIVE_INITIALIZED → JOB_CREATED → JOB_STARTED → JOB_COMPLETED → DRIVE_EJECT_PREPARED</t>
+          <t>Files created and checksums recorded in case-001.sha256</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr"/>
-      <c r="H42" s="5" t="inlineStr"/>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>See section 12.6 step 1 for commands</t>
+        </is>
+      </c>
       <c r="I42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>12.7 Error Handling</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="n"/>
-      <c r="C43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n"/>
-      <c r="G43" s="3" t="n"/>
-      <c r="H43" s="3" t="n"/>
-      <c r="I43" s="4" t="n"/>
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>TC-602</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>E2E: Add mount</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>POST /mounts with local_mount_point: /mnt/test-evidence</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>200, mount created</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr"/>
+      <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>ERR-001</t>
+          <t>TC-603</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Non-existent job returns 404</t>
+          <t>E2E: Discover drive</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
@@ -1782,12 +1817,12 @@
       <c r="D44" s="5" t="inlineStr"/>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>1. GET /jobs/99999</t>
+          <t>Plug USB drive, wait 30s, GET /drives</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>404, NOT_FOUND</t>
+          <t>Drive appears as AVAILABLE</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr"/>
@@ -1797,12 +1832,12 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>ERR-002</t>
+          <t>TC-604</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Non-existent mount returns 404</t>
+          <t>E2E: Initialize drive</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
@@ -1813,12 +1848,12 @@
       <c r="D45" s="5" t="inlineStr"/>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>1. DELETE /mounts/99999</t>
+          <t>POST /drives/{id}/initialize with project_id: PROJ-E2E</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>404, NOT_FOUND</t>
+          <t>200, state → IN_USE</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr"/>
@@ -1828,12 +1863,12 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>ERR-003</t>
+          <t>TC-605</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Start already-running job returns 409</t>
+          <t>E2E: Create job</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -1844,12 +1879,12 @@
       <c r="D46" s="5" t="inlineStr"/>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>1. Start a job that is already RUNNING</t>
+          <t>POST /jobs with source_path pointing to test files</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>409, CONFLICT</t>
+          <t>200, job created</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr"/>
@@ -1859,12 +1894,12 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>ERR-004</t>
+          <t>TC-606</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Error response format</t>
+          <t>E2E: Start job</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -1875,32 +1910,360 @@
       <c r="D47" s="5" t="inlineStr"/>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>1. Trigger any error response
-2. Inspect JSON body</t>
+          <t>POST /jobs/{id}/start</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>JSON body includes code, message, and trace_id</t>
+          <t>200, status → IN_PROGRESS</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr"/>
       <c r="H47" s="5" t="inlineStr"/>
       <c r="I47" s="5" t="inlineStr"/>
     </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>TC-607</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>E2E: Poll until completed</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr"/>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>GET /jobs/{id} repeatedly</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>status becomes COMPLETED</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr"/>
+      <c r="H48" s="5" t="inlineStr"/>
+      <c r="I48" s="5" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>TC-608</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>E2E: Verify checksums</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr"/>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>POST /jobs/{id}/verify</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>All files pass verification</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr"/>
+      <c r="H49" s="5" t="inlineStr"/>
+      <c r="I49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>TC-609</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>E2E: Generate manifest</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr"/>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>POST /jobs/{id}/manifest</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>200, manifest generated</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr"/>
+      <c r="H50" s="5" t="inlineStr"/>
+      <c r="I50" s="5" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>TC-610</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>E2E: Prepare eject</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>POST /drives/{id}/prepare-eject</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>200, state → AVAILABLE</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr"/>
+      <c r="H51" s="5" t="inlineStr"/>
+      <c r="I51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>TC-611</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>E2E: Verify data on another computer</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr"/>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Remove drive, mount on verification computer, compare sha256sums</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>sha256sum diff shows no differences</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr"/>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Compare against case-001.sha256 from step 1</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>TC-612</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>E2E: Audit trail completeness</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr"/>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>GET /audit</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Chain: MOUNT_ADDED → DRIVE_INITIALIZED → JOB_CREATED → JOB_STARTED → JOB_COMPLETED → DRIVE_EJECT_PREPARED</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr"/>
+      <c r="H53" s="5" t="inlineStr"/>
+      <c r="I53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>12.7 Error Handling</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="n"/>
+      <c r="C54" s="3" t="n"/>
+      <c r="D54" s="3" t="n"/>
+      <c r="E54" s="3" t="n"/>
+      <c r="F54" s="3" t="n"/>
+      <c r="G54" s="3" t="n"/>
+      <c r="H54" s="3" t="n"/>
+      <c r="I54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>TC-701</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>GET non-existent job</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr"/>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>GET /jobs/99999</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>404, NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr"/>
+      <c r="H55" s="5" t="inlineStr"/>
+      <c r="I55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>TC-702</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>DELETE non-existent mount</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>DELETE /mounts/99999</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>404, NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr"/>
+      <c r="H56" s="5" t="inlineStr"/>
+      <c r="I56" s="5" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>TC-703</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Start already-running job</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr"/>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>POST /jobs/{id}/start on a running job</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>409, CONFLICT</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr"/>
+      <c r="H57" s="5" t="inlineStr"/>
+      <c r="I57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>TC-704</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Error response format</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Inspect any error response body</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>JSON body includes code, message, and trace_id</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr"/>
+      <c r="H58" s="5" t="inlineStr"/>
+      <c r="I58" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I47"/>
+  <autoFilter ref="A1:I58"/>
   <mergeCells count="7">
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A29:I29"/>
     <mergeCell ref="A25:I25"/>
-    <mergeCell ref="A43:I43"/>
     <mergeCell ref="A41:I41"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A34:I34"/>
+    <mergeCell ref="A54:I54"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C3 C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C16 C17 C18 C19 C20 C21 C22 C23 C24 C26 C27 C28 C30 C31 C32 C33 C35 C36 C37 C38 C39 C40 C42 C44 C45 C46 C47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Status" error="Please select PASS, FAIL, BLOCKED, or NOT RUN" type="list">
+    <dataValidation sqref="C3 C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C16 C17 C18 C19 C20 C21 C22 C23 C24 C26 C27 C28 C30 C31 C32 C33 C35 C36 C37 C38 C39 C40 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C55 C56 C57 C58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid status" error="Pick PASS, FAIL, BLOCKED, or NOT RUN" type="list">
       <formula1>"PASS,FAIL,BLOCKED,NOT RUN"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add OS user and group management endpoints to QA testing guide and update test cases
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,13 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -80,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -91,6 +98,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2467,14 +2478,1200 @@
       <c r="H67" s="3" t="n"/>
       <c r="I67" s="3" t="n"/>
     </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>§12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="n"/>
+      <c r="D68" s="7" t="n"/>
+      <c r="E68" s="7" t="n"/>
+      <c r="F68" s="7" t="n"/>
+      <c r="G68" s="7" t="n"/>
+      <c r="H68" s="7" t="n"/>
+      <c r="I68" s="7" t="n"/>
+    </row>
     <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>TC-901</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>Create group</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/os-groups with {"name": "ecube-testers"}</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>201, returns name, gid, members</t>
+        </is>
+      </c>
+      <c r="F69" s="8" t="n"/>
+      <c r="G69" s="8" t="n"/>
+      <c r="H69" s="8" t="n"/>
+      <c r="I69" s="8" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>TC-902</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>Create group without prefix</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/os-groups with {"name": "testers"}</t>
+        </is>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>422, group name must start with ecube-</t>
+        </is>
+      </c>
+      <c r="F70" s="8" t="n"/>
+      <c r="G70" s="8" t="n"/>
+      <c r="H70" s="8" t="n"/>
+      <c r="I70" s="8" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>TC-903</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>List groups</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>GET /admin/os-groups</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>200, only ecube-* groups listed</t>
+        </is>
+      </c>
+      <c r="F71" s="8" t="n"/>
+      <c r="G71" s="8" t="n"/>
+      <c r="H71" s="8" t="n"/>
+      <c r="I71" s="8" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
+          <t>TC-904</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>Delete group</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>DELETE /admin/os-groups/ecube-testers</t>
+        </is>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F72" s="8" t="n"/>
+      <c r="G72" s="8" t="n"/>
+      <c r="H72" s="8" t="n"/>
+      <c r="I72" s="8" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>TC-905</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>Delete group without prefix</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>DELETE /admin/os-groups/somegroup</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>422, group name must start with ecube-</t>
+        </is>
+      </c>
+      <c r="F73" s="8" t="n"/>
+      <c r="G73" s="8" t="n"/>
+      <c r="H73" s="8" t="n"/>
+      <c r="I73" s="8" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
+        <is>
+          <t>TC-906</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t>Create user</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/os-users with username, password, groups, roles</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>201, returns username, uid, gid, home, shell, groups</t>
+        </is>
+      </c>
+      <c r="F74" s="8" t="n"/>
+      <c r="G74" s="8" t="n"/>
+      <c r="H74" s="8" t="n"/>
+      <c r="I74" s="8" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>TC-907</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Create user — duplicate</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/os-users with existing username</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>409, Conflict</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="n"/>
+      <c r="G75" s="8" t="n"/>
+      <c r="H75" s="8" t="n"/>
+      <c r="I75" s="8" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
+        <is>
+          <t>TC-908</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>Create user — reserved name</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/os-users with {"username": "root", ...}</t>
+        </is>
+      </c>
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>422, reserved username</t>
+        </is>
+      </c>
+      <c r="F76" s="8" t="n"/>
+      <c r="G76" s="8" t="n"/>
+      <c r="H76" s="8" t="n"/>
+      <c r="I76" s="8" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
+          <t>TC-909</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Create user — empty password</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/os-users with {"password": "", ...}</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="n"/>
+      <c r="G77" s="8" t="n"/>
+      <c r="H77" s="8" t="n"/>
+      <c r="I77" s="8" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>TC-910</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>Create user — password with newline</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/os-users with password containing \n</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>422, unsafe characters</t>
+        </is>
+      </c>
+      <c r="F78" s="8" t="n"/>
+      <c r="G78" s="8" t="n"/>
+      <c r="H78" s="8" t="n"/>
+      <c r="I78" s="8" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>TC-911</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>Create user — password with colon</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/os-users with password containing :</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>422, unsafe characters</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="n"/>
+      <c r="G79" s="8" t="n"/>
+      <c r="H79" s="8" t="n"/>
+      <c r="I79" s="8" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>TC-912</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>Create user — invalid group</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/os-users with non-existent group in groups list</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>422, group does not exist</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="n"/>
+      <c r="G80" s="8" t="n"/>
+      <c r="H80" s="8" t="n"/>
+      <c r="I80" s="8" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>TC-913</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>List users</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>GET /admin/os-users</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>200, only users in ecube-* groups listed</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="n"/>
+      <c r="G81" s="8" t="n"/>
+      <c r="H81" s="8" t="n"/>
+      <c r="I81" s="8" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>TC-914</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>Reset password</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="n"/>
+      <c r="G82" s="8" t="n"/>
+      <c r="H82" s="8" t="n"/>
+      <c r="I82" s="8" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>TC-915</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Reset password — non-ECUBE user</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>PUT /admin/os-users/postgres/password</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>422, user is not ECUBE-managed</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="n"/>
+      <c r="G83" s="8" t="n"/>
+      <c r="H83" s="8" t="n"/>
+      <c r="I83" s="8" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="inlineStr">
+        <is>
+          <t>TC-916</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>Replace groups</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>200, updated group list</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="n"/>
+      <c r="G84" s="8" t="n"/>
+      <c r="H84" s="8" t="n"/>
+      <c r="I84" s="8" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>TC-917</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Append groups</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>200, updated group list</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="n"/>
+      <c r="G85" s="8" t="n"/>
+      <c r="H85" s="8" t="n"/>
+      <c r="I85" s="8" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>TC-918</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>Modify groups — non-ECUBE user</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>PUT /admin/os-users/www-data/groups</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="inlineStr">
+        <is>
+          <t>422, user is not ECUBE-managed</t>
+        </is>
+      </c>
+      <c r="F86" s="8" t="n"/>
+      <c r="G86" s="8" t="n"/>
+      <c r="H86" s="8" t="n"/>
+      <c r="I86" s="8" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>TC-919</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Delete user</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>DELETE /admin/os-users/{username}</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>200, user and DB roles removed</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="n"/>
+      <c r="G87" s="8" t="n"/>
+      <c r="H87" s="8" t="n"/>
+      <c r="I87" s="8" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>TC-920</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C88" s="8" t="inlineStr">
+        <is>
+          <t>Delete user — non-ECUBE user</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>DELETE /admin/os-users/daemon</t>
+        </is>
+      </c>
+      <c r="E88" s="8" t="inlineStr">
+        <is>
+          <t>422, user is not ECUBE-managed</t>
+        </is>
+      </c>
+      <c r="F88" s="8" t="n"/>
+      <c r="G88" s="8" t="n"/>
+      <c r="H88" s="8" t="n"/>
+      <c r="I88" s="8" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t>TC-921</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>Delete user — not found</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>DELETE /admin/os-users/nonexistent</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="F89" s="8" t="n"/>
+      <c r="G89" s="8" t="n"/>
+      <c r="H89" s="8" t="n"/>
+      <c r="I89" s="8" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t>TC-922</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>Processor cannot access OS endpoints</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>GET /admin/os-users with processor token</t>
+        </is>
+      </c>
+      <c r="E90" s="8" t="inlineStr">
+        <is>
+          <t>403, FORBIDDEN</t>
+        </is>
+      </c>
+      <c r="F90" s="8" t="n"/>
+      <c r="G90" s="8" t="n"/>
+      <c r="H90" s="8" t="n"/>
+      <c r="I90" s="8" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t>TC-923</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>Non-local mode returns 404</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>404, Not Found</t>
+        </is>
+      </c>
+      <c r="F91" s="8" t="n"/>
+      <c r="G91" s="8" t="n"/>
+      <c r="H91" s="8" t="n"/>
+      <c r="I91" s="8" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="inlineStr">
+        <is>
+          <t>TC-924</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t>OS_USER_CREATED audit log</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
+        </is>
+      </c>
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>Audit entry with actor and username</t>
+        </is>
+      </c>
+      <c r="F92" s="8" t="n"/>
+      <c r="G92" s="8" t="n"/>
+      <c r="H92" s="8" t="n"/>
+      <c r="I92" s="8" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="inlineStr">
+        <is>
+          <t>TC-925</t>
+        </is>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>OS_USER_DELETED audit log</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
+        </is>
+      </c>
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>Audit entry with actor and username</t>
+        </is>
+      </c>
+      <c r="F93" s="8" t="n"/>
+      <c r="G93" s="8" t="n"/>
+      <c r="H93" s="8" t="n"/>
+      <c r="I93" s="8" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
+        <is>
+          <t>TC-926</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>OS_PASSWORD_RESET audit log</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="inlineStr">
+        <is>
+          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
+        </is>
+      </c>
+      <c r="E94" s="8" t="inlineStr">
+        <is>
+          <t>Audit entry (no password in details)</t>
+        </is>
+      </c>
+      <c r="F94" s="8" t="n"/>
+      <c r="G94" s="8" t="n"/>
+      <c r="H94" s="8" t="n"/>
+      <c r="I94" s="8" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="inlineStr">
+        <is>
+          <t>TC-927</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>OS_GROUP_CREATED audit log</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
+        </is>
+      </c>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>Audit entry with group name</t>
+        </is>
+      </c>
+      <c r="F95" s="8" t="n"/>
+      <c r="G95" s="8" t="n"/>
+      <c r="H95" s="8" t="n"/>
+      <c r="I95" s="8" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>TC-928</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>OS_GROUP_DELETED audit log</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>Audit entry with group name</t>
+        </is>
+      </c>
+      <c r="F96" s="8" t="n"/>
+      <c r="G96" s="8" t="n"/>
+      <c r="H96" s="8" t="n"/>
+      <c r="I96" s="8" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>§12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="n"/>
+      <c r="D97" s="7" t="n"/>
+      <c r="E97" s="7" t="n"/>
+      <c r="F97" s="7" t="n"/>
+      <c r="G97" s="7" t="n"/>
+      <c r="H97" s="7" t="n"/>
+      <c r="I97" s="7" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>TC-1001</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>Status — not initialized</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>GET /setup/status on fresh database</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>200, {"initialized": false}</t>
+        </is>
+      </c>
+      <c r="F98" s="8" t="n"/>
+      <c r="G98" s="8" t="n"/>
+      <c r="H98" s="8" t="n"/>
+      <c r="I98" s="8" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="8" t="inlineStr">
+        <is>
+          <t>TC-1002</t>
+        </is>
+      </c>
+      <c r="B99" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Initialize</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/initialize with valid username and password</t>
+        </is>
+      </c>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>200, returns message, username, groups_created</t>
+        </is>
+      </c>
+      <c r="F99" s="8" t="n"/>
+      <c r="G99" s="8" t="n"/>
+      <c r="H99" s="8" t="n"/>
+      <c r="I99" s="8" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="8" t="inlineStr">
+        <is>
+          <t>TC-1003</t>
+        </is>
+      </c>
+      <c r="B100" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>Status — initialized</t>
+        </is>
+      </c>
+      <c r="D100" s="8" t="inlineStr">
+        <is>
+          <t>GET /setup/status after initialization</t>
+        </is>
+      </c>
+      <c r="E100" s="8" t="inlineStr">
+        <is>
+          <t>200, {"initialized": true}</t>
+        </is>
+      </c>
+      <c r="F100" s="8" t="n"/>
+      <c r="G100" s="8" t="n"/>
+      <c r="H100" s="8" t="n"/>
+      <c r="I100" s="8" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="8" t="inlineStr">
+        <is>
+          <t>TC-1004</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>Re-initialize rejected</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/initialize again</t>
+        </is>
+      </c>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>409, Conflict</t>
+        </is>
+      </c>
+      <c r="F101" s="8" t="n"/>
+      <c r="G101" s="8" t="n"/>
+      <c r="H101" s="8" t="n"/>
+      <c r="I101" s="8" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t>TC-1005</t>
+        </is>
+      </c>
+      <c r="B102" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>Invalid username</t>
+        </is>
+      </c>
+      <c r="D102" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/initialize with uppercase or special chars</t>
+        </is>
+      </c>
+      <c r="E102" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="F102" s="8" t="n"/>
+      <c r="G102" s="8" t="n"/>
+      <c r="H102" s="8" t="n"/>
+      <c r="I102" s="8" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>TC-1006</t>
+        </is>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>Empty password</t>
+        </is>
+      </c>
+      <c r="D103" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/initialize with {"password": ""}</t>
+        </is>
+      </c>
+      <c r="E103" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="F103" s="8" t="n"/>
+      <c r="G103" s="8" t="n"/>
+      <c r="H103" s="8" t="n"/>
+      <c r="I103" s="8" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
+        <is>
+          <t>TC-1007</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>Unsafe password chars</t>
+        </is>
+      </c>
+      <c r="D104" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/initialize with password containing newline or colon</t>
+        </is>
+      </c>
+      <c r="E104" s="8" t="inlineStr">
+        <is>
+          <t>422, unsafe characters</t>
+        </is>
+      </c>
+      <c r="F104" s="8" t="n"/>
+      <c r="G104" s="8" t="n"/>
+      <c r="H104" s="8" t="n"/>
+      <c r="I104" s="8" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>TC-1008</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>Login as initialized admin</t>
+        </is>
+      </c>
+      <c r="D105" s="8" t="inlineStr">
+        <is>
+          <t>POST /auth/token with admin credentials from initialization</t>
+        </is>
+      </c>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>200, JWT contains admin role</t>
+        </is>
+      </c>
+      <c r="F105" s="8" t="n"/>
+      <c r="G105" s="8" t="n"/>
+      <c r="H105" s="8" t="n"/>
+      <c r="I105" s="8" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>TC-1009</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>SYSTEM_INITIALIZED audit log</t>
+        </is>
+      </c>
+      <c r="D106" s="8" t="inlineStr">
+        <is>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+        </is>
+      </c>
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>Audit entry with actor</t>
+        </is>
+      </c>
+      <c r="F106" s="8" t="n"/>
+      <c r="G106" s="8" t="n"/>
+      <c r="H106" s="8" t="n"/>
+      <c r="I106" s="8" t="n"/>
+    </row>
+    <row r="107"/>
+    <row r="108">
+      <c r="A108" s="9" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B69" s="5" t="n">
-        <v>58</v>
+      <c r="B108" s="9" t="n">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enforce requirement for ecube-* group in user creation and update related documentation and tests
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:I109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2882,17 +2882,17 @@
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>List users</t>
+          <t>Create user — no ecube-* group</t>
         </is>
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>GET /admin/os-users</t>
+          <t>POST /admin/os-users with no groups or only non-ecube-* groups</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>200, only users in ecube-* groups listed</t>
+          <t>422, at least one ecube-* group required</t>
         </is>
       </c>
       <c r="F81" s="8" t="n"/>
@@ -2913,17 +2913,17 @@
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>Reset password</t>
+          <t>List users</t>
         </is>
       </c>
       <c r="D82" s="8" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
+          <t>GET /admin/os-users</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, only users in ecube-* groups listed</t>
         </is>
       </c>
       <c r="F82" s="8" t="n"/>
@@ -2944,17 +2944,17 @@
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>Reset password — non-ECUBE user</t>
+          <t>Reset password</t>
         </is>
       </c>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/postgres/password</t>
+          <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F83" s="8" t="n"/>
@@ -2975,17 +2975,17 @@
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>Replace groups</t>
+          <t>Reset password — non-ECUBE user</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
+          <t>PUT /admin/os-users/postgres/password</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t>200, updated group list</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F84" s="8" t="n"/>
@@ -3006,12 +3006,12 @@
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>Append groups</t>
+          <t>Replace groups</t>
         </is>
       </c>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
@@ -3037,17 +3037,17 @@
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>Modify groups — non-ECUBE user</t>
+          <t>Append groups</t>
         </is>
       </c>
       <c r="D86" s="8" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/www-data/groups</t>
+          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>200, updated group list</t>
         </is>
       </c>
       <c r="F86" s="8" t="n"/>
@@ -3068,17 +3068,17 @@
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Delete user</t>
+          <t>Modify groups — non-ECUBE user</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/{username}</t>
+          <t>PUT /admin/os-users/www-data/groups</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>200, user and DB roles removed</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F87" s="8" t="n"/>
@@ -3099,17 +3099,17 @@
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>Delete user — non-ECUBE user</t>
+          <t>Delete user</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/daemon</t>
+          <t>DELETE /admin/os-users/{username}</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
+          <t>200, user and DB roles removed</t>
         </is>
       </c>
       <c r="F88" s="8" t="n"/>
@@ -3130,17 +3130,17 @@
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>Delete user — not found</t>
+          <t>Delete user — non-ECUBE user</t>
         </is>
       </c>
       <c r="D89" s="8" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/nonexistent</t>
+          <t>DELETE /admin/os-users/daemon</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F89" s="8" t="n"/>
@@ -3161,17 +3161,17 @@
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Processor cannot access OS endpoints</t>
+          <t>Delete user — not found</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr">
         <is>
-          <t>GET /admin/os-users with processor token</t>
+          <t>DELETE /admin/os-users/nonexistent</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>404</t>
         </is>
       </c>
       <c r="F90" s="8" t="n"/>
@@ -3192,17 +3192,17 @@
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>Non-local mode returns 404</t>
+          <t>Processor cannot access OS endpoints</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
+          <t>GET /admin/os-users with processor token</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>404, Not Found</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F91" s="8" t="n"/>
@@ -3223,17 +3223,17 @@
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>OS_USER_CREATED audit log</t>
+          <t>Non-local mode returns 404</t>
         </is>
       </c>
       <c r="D92" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
+          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>404, Not Found</t>
         </is>
       </c>
       <c r="F92" s="8" t="n"/>
@@ -3254,12 +3254,12 @@
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>OS_USER_DELETED audit log</t>
+          <t>OS_USER_CREATED audit log</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
+          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -3285,17 +3285,17 @@
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t>OS_PASSWORD_RESET audit log</t>
+          <t>OS_USER_DELETED audit log</t>
         </is>
       </c>
       <c r="D94" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
+          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t>Audit entry (no password in details)</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F94" s="8" t="n"/>
@@ -3316,17 +3316,17 @@
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t>OS_GROUP_CREATED audit log</t>
+          <t>OS_PASSWORD_RESET audit log</t>
         </is>
       </c>
       <c r="D95" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
+          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>Audit entry (no password in details)</t>
         </is>
       </c>
       <c r="F95" s="8" t="n"/>
@@ -3347,12 +3347,12 @@
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>OS_GROUP_DELETED audit log</t>
+          <t>OS_GROUP_CREATED audit log</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
+          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
@@ -3366,59 +3366,59 @@
       <c r="I96" s="8" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="6" t="inlineStr">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>TC-929</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>OS_GROUP_DELETED audit log</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>Audit entry with group name</t>
+        </is>
+      </c>
+      <c r="F97" s="8" t="n"/>
+      <c r="G97" s="8" t="n"/>
+      <c r="H97" s="8" t="n"/>
+      <c r="I97" s="8" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="inlineStr">
         <is>
           <t>§12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="B97" s="6" t="inlineStr">
+      <c r="B98" s="6" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C97" s="7" t="n"/>
-      <c r="D97" s="7" t="n"/>
-      <c r="E97" s="7" t="n"/>
-      <c r="F97" s="7" t="n"/>
-      <c r="G97" s="7" t="n"/>
-      <c r="H97" s="7" t="n"/>
-      <c r="I97" s="7" t="n"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="8" t="inlineStr">
-        <is>
-          <t>TC-1001</t>
-        </is>
-      </c>
-      <c r="B98" s="8" t="inlineStr">
-        <is>
-          <t>12.10 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C98" s="8" t="inlineStr">
-        <is>
-          <t>Status — not initialized</t>
-        </is>
-      </c>
-      <c r="D98" s="8" t="inlineStr">
-        <is>
-          <t>GET /setup/status on fresh database</t>
-        </is>
-      </c>
-      <c r="E98" s="8" t="inlineStr">
-        <is>
-          <t>200, {"initialized": false}</t>
-        </is>
-      </c>
-      <c r="F98" s="8" t="n"/>
-      <c r="G98" s="8" t="n"/>
-      <c r="H98" s="8" t="n"/>
-      <c r="I98" s="8" t="n"/>
+      <c r="C98" s="7" t="n"/>
+      <c r="D98" s="7" t="n"/>
+      <c r="E98" s="7" t="n"/>
+      <c r="F98" s="7" t="n"/>
+      <c r="G98" s="7" t="n"/>
+      <c r="H98" s="7" t="n"/>
+      <c r="I98" s="7" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>TC-1002</t>
+          <t>TC-1001</t>
         </is>
       </c>
       <c r="B99" s="8" t="inlineStr">
@@ -3428,17 +3428,17 @@
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t>Initialize</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D99" s="8" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with valid username and password</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t>200, returns message, username, groups_created</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F99" s="8" t="n"/>
@@ -3449,7 +3449,7 @@
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t>TC-1003</t>
+          <t>TC-1002</t>
         </is>
       </c>
       <c r="B100" s="8" t="inlineStr">
@@ -3459,17 +3459,17 @@
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>Status — initialized</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D100" s="8" t="inlineStr">
         <is>
-          <t>GET /setup/status after initialization</t>
+          <t>POST /setup/initialize with valid username and password</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
         <is>
-          <t>200, {"initialized": true}</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F100" s="8" t="n"/>
@@ -3480,7 +3480,7 @@
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>TC-1004</t>
+          <t>TC-1003</t>
         </is>
       </c>
       <c r="B101" s="8" t="inlineStr">
@@ -3490,17 +3490,17 @@
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t>Re-initialize rejected</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F101" s="8" t="n"/>
@@ -3511,7 +3511,7 @@
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t>TC-1005</t>
+          <t>TC-1004</t>
         </is>
       </c>
       <c r="B102" s="8" t="inlineStr">
@@ -3521,17 +3521,17 @@
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>Re-initialize rejected</t>
         </is>
       </c>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>409, Conflict</t>
         </is>
       </c>
       <c r="F102" s="8" t="n"/>
@@ -3542,7 +3542,7 @@
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t>TC-1006</t>
+          <t>TC-1005</t>
         </is>
       </c>
       <c r="B103" s="8" t="inlineStr">
@@ -3552,12 +3552,12 @@
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -3573,7 +3573,7 @@
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t>TC-1007</t>
+          <t>TC-1006</t>
         </is>
       </c>
       <c r="B104" s="8" t="inlineStr">
@@ -3583,17 +3583,17 @@
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F104" s="8" t="n"/>
@@ -3604,7 +3604,7 @@
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t>TC-1008</t>
+          <t>TC-1007</t>
         </is>
       </c>
       <c r="B105" s="8" t="inlineStr">
@@ -3614,17 +3614,17 @@
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>Unsafe password chars</t>
         </is>
       </c>
       <c r="D105" s="8" t="inlineStr">
         <is>
-          <t>POST /auth/token with admin credentials from initialization</t>
+          <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F105" s="8" t="n"/>
@@ -3635,7 +3635,7 @@
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t>TC-1009</t>
+          <t>TC-1008</t>
         </is>
       </c>
       <c r="B106" s="8" t="inlineStr">
@@ -3645,17 +3645,17 @@
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>Login as initialized admin</t>
         </is>
       </c>
       <c r="D106" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>POST /auth/token with admin credentials from initialization</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>200, JWT contains admin role</t>
         </is>
       </c>
       <c r="F106" s="8" t="n"/>
@@ -3663,14 +3663,45 @@
       <c r="H106" s="8" t="n"/>
       <c r="I106" s="8" t="n"/>
     </row>
-    <row r="107"/>
-    <row r="108">
-      <c r="A108" s="9" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>TC-1009</t>
+        </is>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>SYSTEM_INITIALIZED audit log</t>
+        </is>
+      </c>
+      <c r="D107" s="8" t="inlineStr">
+        <is>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+        </is>
+      </c>
+      <c r="E107" s="8" t="inlineStr">
+        <is>
+          <t>Audit entry with actor</t>
+        </is>
+      </c>
+      <c r="F107" s="8" t="n"/>
+      <c r="G107" s="8" t="n"/>
+      <c r="H107" s="8" t="n"/>
+      <c r="I107" s="8" t="n"/>
+    </row>
+    <row r="108"/>
+    <row r="109">
+      <c r="A109" s="9" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B108" s="9" t="n">
+      <c r="B109" s="9" t="n">
         <v>95</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance group management to preserve non-ECUBE groups and enforce ECUBE group requirements in API
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I109"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>200, updated group list</t>
+          <t>200, updated group list; non-ecube-* groups preserved</t>
         </is>
       </c>
       <c r="F85" s="8" t="n"/>
@@ -3037,23 +3037,19 @@
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>Append groups</t>
+          <t>Replace groups — empty list</t>
         </is>
       </c>
       <c r="D86" s="8" t="inlineStr">
         <is>
-          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": []}</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t>200, updated group list</t>
-        </is>
-      </c>
-      <c r="F86" s="8" t="n"/>
-      <c r="G86" s="8" t="n"/>
-      <c r="H86" s="8" t="n"/>
-      <c r="I86" s="8" t="n"/>
+          <t>422, at least one ecube-* group required</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
@@ -3068,23 +3064,19 @@
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Modify groups — non-ECUBE user</t>
+          <t>Replace groups — non-ecube name</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr">
         <is>
-          <t>PUT /admin/os-users/www-data/groups</t>
+          <t>PUT /admin/os-users/{username}/groups with {"groups": ["docker"]}</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>422, user is not ECUBE-managed</t>
-        </is>
-      </c>
-      <c r="F87" s="8" t="n"/>
-      <c r="G87" s="8" t="n"/>
-      <c r="H87" s="8" t="n"/>
-      <c r="I87" s="8" t="n"/>
+          <t>422, group does not start with ecube-</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
@@ -3099,17 +3091,17 @@
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>Delete user</t>
+          <t>Append groups</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/{username}</t>
+          <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t>200, user and DB roles removed</t>
+          <t>200, updated group list</t>
         </is>
       </c>
       <c r="F88" s="8" t="n"/>
@@ -3130,12 +3122,12 @@
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>Delete user — non-ECUBE user</t>
+          <t>Modify groups — non-ECUBE user</t>
         </is>
       </c>
       <c r="D89" s="8" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/daemon</t>
+          <t>PUT /admin/os-users/www-data/groups</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
@@ -3161,17 +3153,17 @@
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Delete user — not found</t>
+          <t>Delete user</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr">
         <is>
-          <t>DELETE /admin/os-users/nonexistent</t>
+          <t>DELETE /admin/os-users/{username}</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t>404</t>
+          <t>200, user and DB roles removed</t>
         </is>
       </c>
       <c r="F90" s="8" t="n"/>
@@ -3192,17 +3184,17 @@
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>Processor cannot access OS endpoints</t>
+          <t>Delete user — non-ECUBE user</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>GET /admin/os-users with processor token</t>
+          <t>DELETE /admin/os-users/daemon</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>403, FORBIDDEN</t>
+          <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
       <c r="F91" s="8" t="n"/>
@@ -3223,17 +3215,17 @@
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>Non-local mode returns 404</t>
+          <t>Delete user — not found</t>
         </is>
       </c>
       <c r="D92" s="8" t="inlineStr">
         <is>
-          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
+          <t>DELETE /admin/os-users/nonexistent</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t>404, Not Found</t>
+          <t>404</t>
         </is>
       </c>
       <c r="F92" s="8" t="n"/>
@@ -3254,17 +3246,17 @@
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>OS_USER_CREATED audit log</t>
+          <t>Processor cannot access OS endpoints</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
+          <t>GET /admin/os-users with processor token</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>403, FORBIDDEN</t>
         </is>
       </c>
       <c r="F93" s="8" t="n"/>
@@ -3285,17 +3277,17 @@
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t>OS_USER_DELETED audit log</t>
+          <t>Non-local mode returns 404</t>
         </is>
       </c>
       <c r="D94" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
+          <t>All /admin/os-* endpoints when role_resolver != "local"</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t>Audit entry with actor and username</t>
+          <t>404, Not Found</t>
         </is>
       </c>
       <c r="F94" s="8" t="n"/>
@@ -3316,17 +3308,17 @@
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t>OS_PASSWORD_RESET audit log</t>
+          <t>OS_USER_CREATED audit log</t>
         </is>
       </c>
       <c r="D95" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
+          <t>GET /audit?action=OS_USER_CREATED after creating user</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t>Audit entry (no password in details)</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F95" s="8" t="n"/>
@@ -3347,17 +3339,17 @@
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>OS_GROUP_CREATED audit log</t>
+          <t>OS_USER_DELETED audit log</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
+          <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>Audit entry with actor and username</t>
         </is>
       </c>
       <c r="F96" s="8" t="n"/>
@@ -3378,17 +3370,17 @@
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>OS_GROUP_DELETED audit log</t>
+          <t>OS_PASSWORD_RESET audit log</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
+          <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t>Audit entry with group name</t>
+          <t>Audit entry (no password in details)</t>
         </is>
       </c>
       <c r="F97" s="8" t="n"/>
@@ -3397,48 +3389,60 @@
       <c r="I97" s="8" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="6" t="inlineStr">
-        <is>
-          <t>§12.10 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>12.10 First-Run Setup</t>
-        </is>
-      </c>
-      <c r="C98" s="7" t="n"/>
-      <c r="D98" s="7" t="n"/>
-      <c r="E98" s="7" t="n"/>
-      <c r="F98" s="7" t="n"/>
-      <c r="G98" s="7" t="n"/>
-      <c r="H98" s="7" t="n"/>
-      <c r="I98" s="7" t="n"/>
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>TC-930</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>12.9 OS User &amp; Group Mgmt</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>OS_GROUP_CREATED audit log</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>Audit entry with group name</t>
+        </is>
+      </c>
+      <c r="F98" s="8" t="n"/>
+      <c r="G98" s="8" t="n"/>
+      <c r="H98" s="8" t="n"/>
+      <c r="I98" s="8" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>TC-1001</t>
+          <t>TC-931</t>
         </is>
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>12.10 First-Run Setup</t>
+          <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t>Status — not initialized</t>
+          <t>OS_GROUP_DELETED audit log</t>
         </is>
       </c>
       <c r="D99" s="8" t="inlineStr">
         <is>
-          <t>GET /setup/status on fresh database</t>
+          <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t>200, {"initialized": false}</t>
+          <t>Audit entry with group name</t>
         </is>
       </c>
       <c r="F99" s="8" t="n"/>
@@ -3447,40 +3451,28 @@
       <c r="I99" s="8" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="8" t="inlineStr">
-        <is>
-          <t>TC-1002</t>
-        </is>
-      </c>
-      <c r="B100" s="8" t="inlineStr">
+      <c r="A100" s="6" t="inlineStr">
+        <is>
+          <t>§12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C100" s="8" t="inlineStr">
-        <is>
-          <t>Initialize</t>
-        </is>
-      </c>
-      <c r="D100" s="8" t="inlineStr">
-        <is>
-          <t>POST /setup/initialize with valid username and password</t>
-        </is>
-      </c>
-      <c r="E100" s="8" t="inlineStr">
-        <is>
-          <t>200, returns message, username, groups_created</t>
-        </is>
-      </c>
-      <c r="F100" s="8" t="n"/>
-      <c r="G100" s="8" t="n"/>
-      <c r="H100" s="8" t="n"/>
-      <c r="I100" s="8" t="n"/>
+      <c r="C100" s="7" t="n"/>
+      <c r="D100" s="7" t="n"/>
+      <c r="E100" s="7" t="n"/>
+      <c r="F100" s="7" t="n"/>
+      <c r="G100" s="7" t="n"/>
+      <c r="H100" s="7" t="n"/>
+      <c r="I100" s="7" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>TC-1003</t>
+          <t>TC-1001</t>
         </is>
       </c>
       <c r="B101" s="8" t="inlineStr">
@@ -3490,17 +3482,17 @@
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t>Status — initialized</t>
+          <t>Status — not initialized</t>
         </is>
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>GET /setup/status after initialization</t>
+          <t>GET /setup/status on fresh database</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
         <is>
-          <t>200, {"initialized": true}</t>
+          <t>200, {"initialized": false}</t>
         </is>
       </c>
       <c r="F101" s="8" t="n"/>
@@ -3511,7 +3503,7 @@
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t>TC-1004</t>
+          <t>TC-1002</t>
         </is>
       </c>
       <c r="B102" s="8" t="inlineStr">
@@ -3521,17 +3513,17 @@
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Re-initialize rejected</t>
+          <t>Initialize</t>
         </is>
       </c>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>POST /setup/initialize again</t>
+          <t>POST /setup/initialize with valid username and password</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t>409, Conflict</t>
+          <t>200, returns message, username, groups_created</t>
         </is>
       </c>
       <c r="F102" s="8" t="n"/>
@@ -3542,7 +3534,7 @@
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t>TC-1005</t>
+          <t>TC-1003</t>
         </is>
       </c>
       <c r="B103" s="8" t="inlineStr">
@@ -3552,17 +3544,17 @@
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Invalid username</t>
+          <t>Status — initialized</t>
         </is>
       </c>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with uppercase or special chars</t>
+          <t>GET /setup/status after initialization</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>200, {"initialized": true}</t>
         </is>
       </c>
       <c r="F103" s="8" t="n"/>
@@ -3573,7 +3565,7 @@
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t>TC-1006</t>
+          <t>TC-1004</t>
         </is>
       </c>
       <c r="B104" s="8" t="inlineStr">
@@ -3583,17 +3575,17 @@
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>Empty password</t>
+          <t>Re-initialize rejected</t>
         </is>
       </c>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with {"password": ""}</t>
+          <t>POST /setup/initialize again</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>409, Conflict</t>
         </is>
       </c>
       <c r="F104" s="8" t="n"/>
@@ -3604,7 +3596,7 @@
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t>TC-1007</t>
+          <t>TC-1005</t>
         </is>
       </c>
       <c r="B105" s="8" t="inlineStr">
@@ -3614,17 +3606,17 @@
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t>Unsafe password chars</t>
+          <t>Invalid username</t>
         </is>
       </c>
       <c r="D105" s="8" t="inlineStr">
         <is>
-          <t>POST /setup/initialize with password containing newline or colon</t>
+          <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
         <is>
-          <t>422, unsafe characters</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F105" s="8" t="n"/>
@@ -3635,7 +3627,7 @@
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t>TC-1008</t>
+          <t>TC-1006</t>
         </is>
       </c>
       <c r="B106" s="8" t="inlineStr">
@@ -3645,17 +3637,17 @@
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t>Login as initialized admin</t>
+          <t>Empty password</t>
         </is>
       </c>
       <c r="D106" s="8" t="inlineStr">
         <is>
-          <t>POST /auth/token with admin credentials from initialization</t>
+          <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
         <is>
-          <t>200, JWT contains admin role</t>
+          <t>422</t>
         </is>
       </c>
       <c r="F106" s="8" t="n"/>
@@ -3666,7 +3658,7 @@
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t>TC-1009</t>
+          <t>TC-1007</t>
         </is>
       </c>
       <c r="B107" s="8" t="inlineStr">
@@ -3676,17 +3668,17 @@
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t>SYSTEM_INITIALIZED audit log</t>
+          <t>Unsafe password chars</t>
         </is>
       </c>
       <c r="D107" s="8" t="inlineStr">
         <is>
-          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+          <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
         <is>
-          <t>Audit entry with actor</t>
+          <t>422, unsafe characters</t>
         </is>
       </c>
       <c r="F107" s="8" t="n"/>
@@ -3694,14 +3686,76 @@
       <c r="H107" s="8" t="n"/>
       <c r="I107" s="8" t="n"/>
     </row>
-    <row r="108"/>
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
+        <is>
+          <t>TC-1008</t>
+        </is>
+      </c>
+      <c r="B108" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>Login as initialized admin</t>
+        </is>
+      </c>
+      <c r="D108" s="8" t="inlineStr">
+        <is>
+          <t>POST /auth/token with admin credentials from initialization</t>
+        </is>
+      </c>
+      <c r="E108" s="8" t="inlineStr">
+        <is>
+          <t>200, JWT contains admin role</t>
+        </is>
+      </c>
+      <c r="F108" s="8" t="n"/>
+      <c r="G108" s="8" t="n"/>
+      <c r="H108" s="8" t="n"/>
+      <c r="I108" s="8" t="n"/>
+    </row>
     <row r="109">
-      <c r="A109" s="9" t="inlineStr">
+      <c r="A109" s="8" t="inlineStr">
+        <is>
+          <t>TC-1009</t>
+        </is>
+      </c>
+      <c r="B109" s="8" t="inlineStr">
+        <is>
+          <t>12.10 First-Run Setup</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>SYSTEM_INITIALIZED audit log</t>
+        </is>
+      </c>
+      <c r="D109" s="8" t="inlineStr">
+        <is>
+          <t>GET /audit?action=SYSTEM_INITIALIZED</t>
+        </is>
+      </c>
+      <c r="E109" s="8" t="inlineStr">
+        <is>
+          <t>Audit entry with actor</t>
+        </is>
+      </c>
+      <c r="F109" s="8" t="n"/>
+      <c r="G109" s="8" t="n"/>
+      <c r="H109" s="8" t="n"/>
+      <c r="I109" s="8" t="n"/>
+    </row>
+    <row r="110"/>
+    <row r="111">
+      <c r="A111" s="9" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B109" s="9" t="n">
+      <c r="B111" s="9" t="n">
         <v>95</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update operational and QA testing guides with API-based database provisioning details
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I111"/>
+  <dimension ref="A1:I129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3748,15 +3748,561 @@
       <c r="H109" s="8" t="n"/>
       <c r="I109" s="8" t="n"/>
     </row>
-    <row r="110"/>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>§12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C110" s="7" t="n"/>
+      <c r="D110" s="7" t="n"/>
+      <c r="E110" s="7" t="n"/>
+      <c r="F110" s="7" t="n"/>
+      <c r="G110" s="7" t="n"/>
+      <c r="H110" s="7" t="n"/>
+      <c r="I110" s="7" t="n"/>
+    </row>
     <row r="111">
-      <c r="A111" s="9" t="inlineStr">
+      <c r="A111" s="8" t="inlineStr">
+        <is>
+          <t>TC-1101</t>
+        </is>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>Test connection — success</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
+        </is>
+      </c>
+      <c r="E111" s="8" t="inlineStr">
+        <is>
+          <t>200, {"status": "ok", "server_version": "..."}</t>
+        </is>
+      </c>
+      <c r="F111" s="8" t="n"/>
+      <c r="G111" s="8" t="n"/>
+      <c r="H111" s="8" t="n"/>
+      <c r="I111" s="8" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>TC-1102</t>
+        </is>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>Test connection — bad host</t>
+        </is>
+      </c>
+      <c r="D112" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/test-connection with unreachable host</t>
+        </is>
+      </c>
+      <c r="E112" s="8" t="inlineStr">
+        <is>
+          <t>400, connection error</t>
+        </is>
+      </c>
+      <c r="F112" s="8" t="n"/>
+      <c r="G112" s="8" t="n"/>
+      <c r="H112" s="8" t="n"/>
+      <c r="I112" s="8" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="inlineStr">
+        <is>
+          <t>TC-1103</t>
+        </is>
+      </c>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>Test connection — SSRF host</t>
+        </is>
+      </c>
+      <c r="D113" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
+        </is>
+      </c>
+      <c r="E113" s="8" t="inlineStr">
+        <is>
+          <t>422, invalid host</t>
+        </is>
+      </c>
+      <c r="F113" s="8" t="n"/>
+      <c r="G113" s="8" t="n"/>
+      <c r="H113" s="8" t="n"/>
+      <c r="I113" s="8" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="inlineStr">
+        <is>
+          <t>TC-1104</t>
+        </is>
+      </c>
+      <c r="B114" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>Test connection — port out of range</t>
+        </is>
+      </c>
+      <c r="D114" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/test-connection with "port": 99999</t>
+        </is>
+      </c>
+      <c r="E114" s="8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="F114" s="8" t="n"/>
+      <c r="G114" s="8" t="n"/>
+      <c r="H114" s="8" t="n"/>
+      <c r="I114" s="8" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="8" t="inlineStr">
+        <is>
+          <t>TC-1105</t>
+        </is>
+      </c>
+      <c r="B115" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="inlineStr">
+        <is>
+          <t>Provision — success</t>
+        </is>
+      </c>
+      <c r="D115" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with valid credentials</t>
+        </is>
+      </c>
+      <c r="E115" s="8" t="inlineStr">
+        <is>
+          <t>200, returns database, user, migrations_applied</t>
+        </is>
+      </c>
+      <c r="F115" s="8" t="n"/>
+      <c r="G115" s="8" t="n"/>
+      <c r="H115" s="8" t="n"/>
+      <c r="I115" s="8" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="8" t="inlineStr">
+        <is>
+          <t>TC-1106</t>
+        </is>
+      </c>
+      <c r="B116" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
+          <t>Provision — bad admin credentials</t>
+        </is>
+      </c>
+      <c r="D116" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with wrong admin password</t>
+        </is>
+      </c>
+      <c r="E116" s="8" t="inlineStr">
+        <is>
+          <t>400, connection error</t>
+        </is>
+      </c>
+      <c r="F116" s="8" t="n"/>
+      <c r="G116" s="8" t="n"/>
+      <c r="H116" s="8" t="n"/>
+      <c r="I116" s="8" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
+        <is>
+          <t>TC-1107</t>
+        </is>
+      </c>
+      <c r="B117" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>Provision — invalid database name</t>
+        </is>
+      </c>
+      <c r="D117" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with "app_database": "drop;--"</t>
+        </is>
+      </c>
+      <c r="E117" s="8" t="inlineStr">
+        <is>
+          <t>422, invalid identifier</t>
+        </is>
+      </c>
+      <c r="F117" s="8" t="n"/>
+      <c r="G117" s="8" t="n"/>
+      <c r="H117" s="8" t="n"/>
+      <c r="I117" s="8" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="8" t="inlineStr">
+        <is>
+          <t>TC-1108</t>
+        </is>
+      </c>
+      <c r="B118" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>Status — connected</t>
+        </is>
+      </c>
+      <c r="D118" s="8" t="inlineStr">
+        <is>
+          <t>GET /setup/database/status with admin token</t>
+        </is>
+      </c>
+      <c r="E118" s="8" t="inlineStr">
+        <is>
+          <t>200, connected: true, migration info</t>
+        </is>
+      </c>
+      <c r="F118" s="8" t="n"/>
+      <c r="G118" s="8" t="n"/>
+      <c r="H118" s="8" t="n"/>
+      <c r="I118" s="8" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="8" t="inlineStr">
+        <is>
+          <t>TC-1109</t>
+        </is>
+      </c>
+      <c r="B119" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>Status — requires auth</t>
+        </is>
+      </c>
+      <c r="D119" s="8" t="inlineStr">
+        <is>
+          <t>GET /setup/database/status without token</t>
+        </is>
+      </c>
+      <c r="E119" s="8" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F119" s="8" t="n"/>
+      <c r="G119" s="8" t="n"/>
+      <c r="H119" s="8" t="n"/>
+      <c r="I119" s="8" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
+        <is>
+          <t>TC-1110</t>
+        </is>
+      </c>
+      <c r="B120" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t>Status — requires admin</t>
+        </is>
+      </c>
+      <c r="D120" s="8" t="inlineStr">
+        <is>
+          <t>GET /setup/database/status with processor token</t>
+        </is>
+      </c>
+      <c r="E120" s="8" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="F120" s="8" t="n"/>
+      <c r="G120" s="8" t="n"/>
+      <c r="H120" s="8" t="n"/>
+      <c r="I120" s="8" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="8" t="inlineStr">
+        <is>
+          <t>TC-1111</t>
+        </is>
+      </c>
+      <c r="B121" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>Settings update — success</t>
+        </is>
+      </c>
+      <c r="D121" s="8" t="inlineStr">
+        <is>
+          <t>PUT /setup/database/settings with valid partial update</t>
+        </is>
+      </c>
+      <c r="E121" s="8" t="inlineStr">
+        <is>
+          <t>200, {"status": "updated", ...}</t>
+        </is>
+      </c>
+      <c r="F121" s="8" t="n"/>
+      <c r="G121" s="8" t="n"/>
+      <c r="H121" s="8" t="n"/>
+      <c r="I121" s="8" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="8" t="inlineStr">
+        <is>
+          <t>TC-1112</t>
+        </is>
+      </c>
+      <c r="B122" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>Settings update — bad connection</t>
+        </is>
+      </c>
+      <c r="D122" s="8" t="inlineStr">
+        <is>
+          <t>PUT /setup/database/settings with unreachable host</t>
+        </is>
+      </c>
+      <c r="E122" s="8" t="inlineStr">
+        <is>
+          <t>400, connection test failed</t>
+        </is>
+      </c>
+      <c r="F122" s="8" t="n"/>
+      <c r="G122" s="8" t="n"/>
+      <c r="H122" s="8" t="n"/>
+      <c r="I122" s="8" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="8" t="inlineStr">
+        <is>
+          <t>TC-1113</t>
+        </is>
+      </c>
+      <c r="B123" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C123" s="8" t="inlineStr">
+        <is>
+          <t>Settings update — empty body</t>
+        </is>
+      </c>
+      <c r="D123" s="8" t="inlineStr">
+        <is>
+          <t>PUT /setup/database/settings with {}</t>
+        </is>
+      </c>
+      <c r="E123" s="8" t="inlineStr">
+        <is>
+          <t>422, at least one field required</t>
+        </is>
+      </c>
+      <c r="F123" s="8" t="n"/>
+      <c r="G123" s="8" t="n"/>
+      <c r="H123" s="8" t="n"/>
+      <c r="I123" s="8" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="8" t="inlineStr">
+        <is>
+          <t>TC-1114</t>
+        </is>
+      </c>
+      <c r="B124" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C124" s="8" t="inlineStr">
+        <is>
+          <t>Settings update — requires admin</t>
+        </is>
+      </c>
+      <c r="D124" s="8" t="inlineStr">
+        <is>
+          <t>PUT /setup/database/settings with processor token</t>
+        </is>
+      </c>
+      <c r="E124" s="8" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="F124" s="8" t="n"/>
+      <c r="G124" s="8" t="n"/>
+      <c r="H124" s="8" t="n"/>
+      <c r="I124" s="8" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="8" t="inlineStr">
+        <is>
+          <t>TC-1115</t>
+        </is>
+      </c>
+      <c r="B125" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C125" s="8" t="inlineStr">
+        <is>
+          <t>Auth after setup — test-connection</t>
+        </is>
+      </c>
+      <c r="D125" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/test-connection without token (after admin exists)</t>
+        </is>
+      </c>
+      <c r="E125" s="8" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F125" s="8" t="n"/>
+      <c r="G125" s="8" t="n"/>
+      <c r="H125" s="8" t="n"/>
+      <c r="I125" s="8" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="8" t="inlineStr">
+        <is>
+          <t>TC-1116</t>
+        </is>
+      </c>
+      <c r="B126" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C126" s="8" t="inlineStr">
+        <is>
+          <t>Auth after setup — provision</t>
+        </is>
+      </c>
+      <c r="D126" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision without token (after admin exists)</t>
+        </is>
+      </c>
+      <c r="E126" s="8" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="F126" s="8" t="n"/>
+      <c r="G126" s="8" t="n"/>
+      <c r="H126" s="8" t="n"/>
+      <c r="I126" s="8" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="inlineStr">
+        <is>
+          <t>TC-1117</t>
+        </is>
+      </c>
+      <c r="B127" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C127" s="8" t="inlineStr">
+        <is>
+          <t>Password redaction</t>
+        </is>
+      </c>
+      <c r="D127" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision and check response</t>
+        </is>
+      </c>
+      <c r="E127" s="8" t="inlineStr">
+        <is>
+          <t>No password in response body</t>
+        </is>
+      </c>
+      <c r="F127" s="8" t="n"/>
+      <c r="G127" s="8" t="n"/>
+      <c r="H127" s="8" t="n"/>
+      <c r="I127" s="8" t="n"/>
+    </row>
+    <row r="128"/>
+    <row r="129">
+      <c r="A129" s="9" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B111" s="9" t="n">
-        <v>95</v>
+      <c r="B129" s="9" t="n">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add force option to database provisioning and implement conflict handling
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I129"/>
+  <dimension ref="A1:I131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4294,16 +4294,84 @@
       <c r="H127" s="8" t="n"/>
       <c r="I127" s="8" t="n"/>
     </row>
-    <row r="128"/>
+    <row r="128">
+      <c r="A128" s="8" t="inlineStr">
+        <is>
+          <t>TC-1118</t>
+        </is>
+      </c>
+      <c r="B128" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C128" s="8" t="inlineStr">
+        <is>
+          <t>Re-provision blocked</t>
+        </is>
+      </c>
+      <c r="D128" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision after successful provisioning (no force)</t>
+        </is>
+      </c>
+      <c r="E128" s="8" t="inlineStr">
+        <is>
+          <t>409, already provisioned</t>
+        </is>
+      </c>
+      <c r="F128" s="8" t="n"/>
+      <c r="G128" s="8" t="n"/>
+      <c r="H128" s="8" t="n"/>
+      <c r="I128" s="8" t="n"/>
+    </row>
     <row r="129">
-      <c r="A129" s="9" t="inlineStr">
+      <c r="A129" s="8" t="inlineStr">
+        <is>
+          <t>TC-1119</t>
+        </is>
+      </c>
+      <c r="B129" s="8" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t>Force re-provision</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with "force": true after successful provisioning</t>
+        </is>
+      </c>
+      <c r="E129" s="8" t="inlineStr">
+        <is>
+          <t>200, returns database, user, migrations_applied</t>
+        </is>
+      </c>
+      <c r="F129" s="8" t="n"/>
+      <c r="G129" s="8" t="n"/>
+      <c r="H129" s="8" t="n"/>
+      <c r="I129" s="8" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="8" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B129" s="9" t="n">
-        <v>112</v>
-      </c>
+      <c r="B131" s="8" t="n">
+        <v>114</v>
+      </c>
+      <c r="C131" s="8" t="n"/>
+      <c r="D131" s="8" t="n"/>
+      <c r="E131" s="8" t="n"/>
+      <c r="F131" s="8" t="n"/>
+      <c r="G131" s="8" t="n"/>
+      <c r="H131" s="8" t="n"/>
+      <c r="I131" s="8" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>

</xml_diff>

<commit_message>
Implement fail-closed behavior for database provisioning endpoints to return 503 when DB is unreachable and no valid admin JWT is provided; update documentation and add tests for this behavior.
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="QA Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'QA Test Cases'!$A$1:$I$1</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,28 +26,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -62,14 +48,8 @@
         <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E2F3"/>
-        <bgColor rgb="00D9E2F3"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -77,31 +57,21 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,13 +437,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I131"/>
+  <dimension ref="A1:I133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -539,26 +509,26 @@
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>TC-101</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Valid login</t>
         </is>
@@ -570,26 +540,26 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>200, access_token and token_type: bearer</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
+          <t>200, response contains access_token and token_type: "bearer"</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TC-102</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Invalid password</t>
         </is>
@@ -604,23 +574,23 @@
           <t>401, Invalid credentials</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>TC-103</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Unknown user</t>
         </is>
@@ -635,23 +605,23 @@
           <t>401, Invalid credentials</t>
         </is>
       </c>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>TC-104</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Missing username</t>
         </is>
@@ -666,23 +636,23 @@
           <t>422</t>
         </is>
       </c>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>TC-105</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Missing password</t>
         </is>
@@ -697,23 +667,23 @@
           <t>422</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>TC-106</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Empty username</t>
         </is>
@@ -728,23 +698,23 @@
           <t>422</t>
         </is>
       </c>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>TC-107</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Token contains correct roles</t>
         </is>
@@ -756,26 +726,26 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>roles matches DB user_roles entry if present, otherwise matches LOCAL_GROUP_ROLE_MAP</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
+          <t>roles matches DB user_roles entry if present, otherwise matches group mapping in LOCAL_GROUP_ROLE_MAP</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>TC-108</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Token contains groups</t>
         </is>
@@ -790,23 +760,23 @@
           <t>groups lists the user's OS groups</t>
         </is>
       </c>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>TC-109</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Token is usable</t>
         </is>
@@ -821,23 +791,23 @@
           <t>200</t>
         </is>
       </c>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>TC-110</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Login audit log</t>
         </is>
@@ -852,23 +822,23 @@
           <t>AUTH_SUCCESS entry with username</t>
         </is>
       </c>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TC-111</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Failed login audit log</t>
         </is>
@@ -883,23 +853,23 @@
           <t>AUTH_FAILURE entry with username</t>
         </is>
       </c>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TC-112</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>12.1 Login Endpoint</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>No auth required for login</t>
         </is>
@@ -914,10 +884,10 @@
           <t>200 (not 401)</t>
         </is>
       </c>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -930,26 +900,26 @@
           <t>12.2 Authorization</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>TC-201</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>12.2 Authorization</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>No token</t>
         </is>
@@ -964,30 +934,30 @@
           <t>401, UNAUTHORIZED</t>
         </is>
       </c>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>TC-202</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>12.2 Authorization</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Garbage token</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Authorization: Bearer not.a.real.token</t>
+          <t>Add header Authorization: Bearer not.a.real.token</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -995,30 +965,30 @@
           <t>401, UNAUTHORIZED</t>
         </is>
       </c>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
+      <c r="F17" s="4" t="n"/>
+      <c r="G17" s="4" t="n"/>
+      <c r="H17" s="4" t="n"/>
+      <c r="I17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>TC-203</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>12.2 Authorization</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Expired token</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Generate token with exp in the past</t>
+          <t>Generate token with 'exp': int(time.time()) - 60</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1026,23 +996,23 @@
           <t>401, UNAUTHORIZED</t>
         </is>
       </c>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>TC-204</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>12.2 Authorization</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Processor adds mount</t>
         </is>
@@ -1057,23 +1027,23 @@
           <t>403, FORBIDDEN</t>
         </is>
       </c>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>TC-205</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>12.2 Authorization</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Processor initializes drive</t>
         </is>
@@ -1088,23 +1058,23 @@
           <t>403, FORBIDDEN</t>
         </is>
       </c>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
+      <c r="F20" s="4" t="n"/>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>TC-206</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>12.2 Authorization</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Processor reads audit</t>
         </is>
@@ -1119,23 +1089,23 @@
           <t>403, FORBIDDEN</t>
         </is>
       </c>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>TC-207</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>12.2 Authorization</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Auditor reads audit</t>
         </is>
@@ -1150,23 +1120,23 @@
           <t>200</t>
         </is>
       </c>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>TC-208</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>12.2 Authorization</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Processor creates job</t>
         </is>
@@ -1181,25 +1151,25 @@
           <t>200</t>
         </is>
       </c>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>TC-209</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>12.2 Authorization</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Error responses have trace_id</t>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>All error responses have trace_id</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1212,10 +1182,10 @@
           <t>trace_id field present</t>
         </is>
       </c>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1228,106 +1198,94 @@
           <t>12.3 Project Isolation</t>
         </is>
       </c>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>TC-301</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>12.3 Project Isolation</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Initialize drive with PROJ-A</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>POST /drives/{id}/initialize with project_id PROJ-A on AVAILABLE drive</t>
-        </is>
-      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Initialize an AVAILABLE drive with PROJ-A</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
           <t>200, state → IN_USE</t>
         </is>
       </c>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>TC-302</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>12.3 Project Isolation</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Cross-project rejection</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>POST /drives/{id}/initialize with project_id PROJ-B on same drive</t>
-        </is>
-      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Re-initialize same drive with PROJ-B</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr">
         <is>
           <t>403, FORBIDDEN — isolation violation</t>
         </is>
       </c>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>TC-303</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>12.3 Project Isolation</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Isolation audit log</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>GET /audit?action=PROJECT_ISOLATION_VIOLATION</t>
-        </is>
-      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Check audit log for PROJECT_ISOLATION_VIOLATION</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Record with requested_project_id: PROJ-B</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
+          <t>Record present with requested_project_id: PROJ-B</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="n"/>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1340,137 +1298,121 @@
           <t>12.4 Drive State Machine</t>
         </is>
       </c>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
+      <c r="G29" s="3" t="n"/>
+      <c r="H29" s="3" t="n"/>
+      <c r="I29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>TC-401</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>12.4 Drive State Machine</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Initialize AVAILABLE drive</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>POST /drives/{id}/initialize on AVAILABLE drive</t>
-        </is>
-      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Initialize an AVAILABLE drive</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
           <t>200, state → IN_USE</t>
         </is>
       </c>
-      <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="3" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>TC-402</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>12.4 Drive State Machine</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Initialize EMPTY drive</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>POST /drives/{id}/initialize on EMPTY drive</t>
-        </is>
-      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Initialize an EMPTY drive</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr">
         <is>
           <t>200, state → IN_USE</t>
         </is>
       </c>
-      <c r="F31" s="3" t="n"/>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="3" t="n"/>
-      <c r="I31" s="3" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>TC-403</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>12.4 Drive State Machine</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Prepare-eject IN_USE drive</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>POST /drives/{id}/prepare-eject on IN_USE drive</t>
-        </is>
-      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Prepare-eject an IN_USE drive</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
           <t>200, state → AVAILABLE</t>
         </is>
       </c>
-      <c r="F32" s="3" t="n"/>
-      <c r="G32" s="3" t="n"/>
-      <c r="H32" s="3" t="n"/>
-      <c r="I32" s="3" t="n"/>
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
+      <c r="I32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>TC-404</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>12.4 Drive State Machine</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Prepare-eject AVAILABLE drive</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>POST /drives/{id}/prepare-eject on AVAILABLE drive</t>
-        </is>
-      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Prepare-eject an AVAILABLE drive</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr">
         <is>
           <t>409, CONFLICT</t>
         </is>
       </c>
-      <c r="F33" s="3" t="n"/>
-      <c r="G33" s="3" t="n"/>
-      <c r="H33" s="3" t="n"/>
-      <c r="I33" s="3" t="n"/>
+      <c r="F33" s="4" t="n"/>
+      <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="n"/>
+      <c r="I33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1483,57 +1425,57 @@
           <t>12.5 USB Hardware</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
+      <c r="C34" s="3" t="n"/>
+      <c r="D34" s="3" t="n"/>
+      <c r="E34" s="3" t="n"/>
+      <c r="F34" s="3" t="n"/>
+      <c r="G34" s="3" t="n"/>
+      <c r="H34" s="3" t="n"/>
+      <c r="I34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>TC-501</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>12.5 USB Hardware</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Hot-plug detection</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Plug in USB drive, wait 30 seconds, GET /drives</t>
+          <t>Plug in a USB drive, wait 30 seconds</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Drive appears in AVAILABLE state</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n"/>
+          <t>GET /drives shows the new drive in AVAILABLE state (discovery auto-transitions EMPTY → AVAILABLE)</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="n"/>
+      <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="n"/>
+      <c r="I35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>TC-502</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>12.5 USB Hardware</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>USB topology</t>
         </is>
@@ -1545,88 +1487,88 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Shows real hub serial numbers, port numbers, devices</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="n"/>
-      <c r="G36" s="3" t="n"/>
-      <c r="H36" s="3" t="n"/>
-      <c r="I36" s="3" t="n"/>
+          <t>Shows real hub serial numbers, port numbers, connected devices</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
+      <c r="I36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>TC-503</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>12.5 USB Hardware</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>Physical eject</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Initialize → prepare-eject → physically remove drive</t>
+          <t>Initialize drive → prepare-eject → physically remove</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Drive listed with current_state=EMPTY; DRIVE_EJECT_PREPARED in audit</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
-      <c r="H37" s="3" t="n"/>
-      <c r="I37" s="3" t="n"/>
+          <t>After the next discovery cycle, GET /drives still lists the drive with current_state=EMPTY; audit shows DRIVE_EJECT_PREPARED</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>TC-504</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>12.5 USB Hardware</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Re-plug same drive</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Remove and re-insert same USB drive</t>
+          <t>Remove and re-insert the same drive</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Drive reappears as AVAILABLE with same device_identifier</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="n"/>
-      <c r="G38" s="3" t="n"/>
-      <c r="H38" s="3" t="n"/>
-      <c r="I38" s="3" t="n"/>
+          <t>Drive reappears as AVAILABLE with same device_identifier (after discovery cycle)</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="n"/>
+      <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
+      <c r="I38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>TC-505</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>12.5 USB Hardware</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Multiple drives</t>
         </is>
@@ -1638,44 +1580,44 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>All drives in /drives; each initializable to different projects</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
-      <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
+          <t>All drives appear in /drives; each can be initialized to different projects</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="n"/>
+      <c r="G39" s="4" t="n"/>
+      <c r="H39" s="4" t="n"/>
+      <c r="I39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>TC-506</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>12.5 USB Hardware</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Sync + unmount</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Initialize → create/start job → prepare-eject</t>
+          <t>Initialize drive, create/start a job, then prepare-eject</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Filesystem flushed and unmounted (verify via mount command)</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="n"/>
-      <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="n"/>
+          <t>Filesystem flushed and unmounted before eject (verify via mount command — no partitions from that drive should be listed)</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="n"/>
+      <c r="G40" s="4" t="n"/>
+      <c r="H40" s="4" t="n"/>
+      <c r="I40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1688,26 +1630,26 @@
           <t>12.6 End-to-End Copy</t>
         </is>
       </c>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
-      <c r="G41" s="2" t="n"/>
-      <c r="H41" s="2" t="n"/>
-      <c r="I41" s="2" t="n"/>
+      <c r="C41" s="3" t="n"/>
+      <c r="D41" s="3" t="n"/>
+      <c r="E41" s="3" t="n"/>
+      <c r="F41" s="3" t="n"/>
+      <c r="G41" s="3" t="n"/>
+      <c r="H41" s="3" t="n"/>
+      <c r="I41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>TC-601</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>12.6 End-to-End Copy</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Full E2E workflow</t>
         </is>
@@ -1722,10 +1664,10 @@
           <t>All steps succeed; checksums match; audit trail shows complete chain</t>
         </is>
       </c>
-      <c r="F42" s="3" t="n"/>
-      <c r="G42" s="3" t="n"/>
-      <c r="H42" s="3" t="n"/>
-      <c r="I42" s="3" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1738,137 +1680,121 @@
           <t>12.7 Error Handling</t>
         </is>
       </c>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="n"/>
+      <c r="C43" s="3" t="n"/>
+      <c r="D43" s="3" t="n"/>
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
+      <c r="I43" s="3" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>TC-701</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>12.7 Error Handling</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Non-existent job</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>GET /jobs/99999</t>
         </is>
       </c>
+      <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
         <is>
           <t>404, NOT_FOUND</t>
         </is>
       </c>
-      <c r="F44" s="3" t="n"/>
-      <c r="G44" s="3" t="n"/>
-      <c r="H44" s="3" t="n"/>
-      <c r="I44" s="3" t="n"/>
+      <c r="F44" s="4" t="n"/>
+      <c r="G44" s="4" t="n"/>
+      <c r="H44" s="4" t="n"/>
+      <c r="I44" s="4" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>TC-702</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>12.7 Error Handling</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Non-existent mount</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>DELETE /mounts/99999</t>
         </is>
       </c>
+      <c r="D45" s="4" t="inlineStr"/>
       <c r="E45" s="4" t="inlineStr">
         <is>
           <t>404, NOT_FOUND</t>
         </is>
       </c>
-      <c r="F45" s="3" t="n"/>
-      <c r="G45" s="3" t="n"/>
-      <c r="H45" s="3" t="n"/>
-      <c r="I45" s="3" t="n"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>TC-703</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>12.7 Error Handling</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>Start already-running job</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>POST /jobs/{id}/start on running job</t>
-        </is>
-      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Start an already-running job</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
           <t>409, CONFLICT</t>
         </is>
       </c>
-      <c r="F46" s="3" t="n"/>
-      <c r="G46" s="3" t="n"/>
-      <c r="H46" s="3" t="n"/>
-      <c r="I46" s="3" t="n"/>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
+      <c r="I46" s="4" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>TC-704</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>12.7 Error Handling</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>Error response format</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Inspect any 4xx/5xx error response</t>
-        </is>
-      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>All error responses</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr"/>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>JSON includes code, message, and trace_id</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="n"/>
-      <c r="G47" s="3" t="n"/>
-      <c r="H47" s="3" t="n"/>
-      <c r="I47" s="3" t="n"/>
+          <t>JSON body includes code, message, and trace_id</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="n"/>
+      <c r="G47" s="4" t="n"/>
+      <c r="H47" s="4" t="n"/>
+      <c r="I47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1881,26 +1807,26 @@
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C48" s="2" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
-      <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="n"/>
+      <c r="C48" s="3" t="n"/>
+      <c r="D48" s="3" t="n"/>
+      <c r="E48" s="3" t="n"/>
+      <c r="F48" s="3" t="n"/>
+      <c r="G48" s="3" t="n"/>
+      <c r="H48" s="3" t="n"/>
+      <c r="I48" s="3" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>TC-801</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>List users (empty)</t>
         </is>
@@ -1915,23 +1841,23 @@
           <t>200, {"users": []}</t>
         </is>
       </c>
-      <c r="F49" s="3" t="n"/>
-      <c r="G49" s="3" t="n"/>
-      <c r="H49" s="3" t="n"/>
-      <c r="I49" s="3" t="n"/>
+      <c r="F49" s="4" t="n"/>
+      <c r="G49" s="4" t="n"/>
+      <c r="H49" s="4" t="n"/>
+      <c r="I49" s="4" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>TC-802</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C50" s="3" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>Assign roles</t>
         </is>
@@ -1946,23 +1872,23 @@
           <t>200, returns username and sorted roles</t>
         </is>
       </c>
-      <c r="F50" s="3" t="n"/>
-      <c r="G50" s="3" t="n"/>
-      <c r="H50" s="3" t="n"/>
-      <c r="I50" s="3" t="n"/>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
+      <c r="I50" s="4" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>TC-803</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Get roles</t>
         </is>
@@ -1977,23 +1903,23 @@
           <t>200, {"username": "qa-processor", "roles": ["auditor", "processor"]}</t>
         </is>
       </c>
-      <c r="F51" s="3" t="n"/>
-      <c r="G51" s="3" t="n"/>
-      <c r="H51" s="3" t="n"/>
-      <c r="I51" s="3" t="n"/>
+      <c r="F51" s="4" t="n"/>
+      <c r="G51" s="4" t="n"/>
+      <c r="H51" s="4" t="n"/>
+      <c r="I51" s="4" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>TC-804</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>List users after assignment</t>
         </is>
@@ -2008,23 +1934,23 @@
           <t>200, user appears in list with correct roles</t>
         </is>
       </c>
-      <c r="F52" s="3" t="n"/>
-      <c r="G52" s="3" t="n"/>
-      <c r="H52" s="3" t="n"/>
-      <c r="I52" s="3" t="n"/>
+      <c r="F52" s="4" t="n"/>
+      <c r="G52" s="4" t="n"/>
+      <c r="H52" s="4" t="n"/>
+      <c r="I52" s="4" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>TC-805</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>Replace roles</t>
         </is>
@@ -2039,30 +1965,30 @@
           <t>200, only ["manager"] returned; old roles removed</t>
         </is>
       </c>
-      <c r="F53" s="3" t="n"/>
-      <c r="G53" s="3" t="n"/>
-      <c r="H53" s="3" t="n"/>
-      <c r="I53" s="3" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="4" t="n"/>
+      <c r="H53" s="4" t="n"/>
+      <c r="I53" s="4" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>TC-806</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>Deduplicate roles</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>PUT with {"roles": ["admin", "admin", "processor"]}</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["admin", "admin", "processor"]}</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
@@ -2070,30 +1996,30 @@
           <t>200, deduplicated to ["admin", "processor"]</t>
         </is>
       </c>
-      <c r="F54" s="3" t="n"/>
-      <c r="G54" s="3" t="n"/>
-      <c r="H54" s="3" t="n"/>
-      <c r="I54" s="3" t="n"/>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="4" t="n"/>
+      <c r="H54" s="4" t="n"/>
+      <c r="I54" s="4" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>TC-807</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>Invalid role name</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>PUT with {"roles": ["superuser"]}</t>
+          <t>PUT /users/qa-processor/roles with {"roles": ["superuser"]}</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
@@ -2101,30 +2027,30 @@
           <t>422, error message mentions superuser</t>
         </is>
       </c>
-      <c r="F55" s="3" t="n"/>
-      <c r="G55" s="3" t="n"/>
-      <c r="H55" s="3" t="n"/>
-      <c r="I55" s="3" t="n"/>
+      <c r="F55" s="4" t="n"/>
+      <c r="G55" s="4" t="n"/>
+      <c r="H55" s="4" t="n"/>
+      <c r="I55" s="4" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>TC-808</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>Empty role list</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>PUT with {"roles": []}</t>
+          <t>PUT /users/qa-processor/roles with {"roles": []}</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -2132,23 +2058,23 @@
           <t>422, at least one role required</t>
         </is>
       </c>
-      <c r="F56" s="3" t="n"/>
-      <c r="G56" s="3" t="n"/>
-      <c r="H56" s="3" t="n"/>
-      <c r="I56" s="3" t="n"/>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="4" t="n"/>
+      <c r="H56" s="4" t="n"/>
+      <c r="I56" s="4" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>TC-809</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>Remove roles</t>
         </is>
@@ -2163,23 +2089,23 @@
           <t>200, {"username": "qa-processor", "roles": []}</t>
         </is>
       </c>
-      <c r="F57" s="3" t="n"/>
-      <c r="G57" s="3" t="n"/>
-      <c r="H57" s="3" t="n"/>
-      <c r="I57" s="3" t="n"/>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
+      <c r="I57" s="4" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>TC-810</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>Get roles after removal</t>
         </is>
@@ -2194,25 +2120,25 @@
           <t>200, {"roles": []}</t>
         </is>
       </c>
-      <c r="F58" s="3" t="n"/>
-      <c r="G58" s="3" t="n"/>
-      <c r="H58" s="3" t="n"/>
-      <c r="I58" s="3" t="n"/>
+      <c r="F58" s="4" t="n"/>
+      <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
+      <c r="I58" s="4" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>TC-811</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>Get roles unknown user</t>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Get roles for unknown user</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -2225,23 +2151,23 @@
           <t>200, {"username": "nonexistent", "roles": []}</t>
         </is>
       </c>
-      <c r="F59" s="3" t="n"/>
-      <c r="G59" s="3" t="n"/>
-      <c r="H59" s="3" t="n"/>
-      <c r="I59" s="3" t="n"/>
+      <c r="F59" s="4" t="n"/>
+      <c r="G59" s="4" t="n"/>
+      <c r="H59" s="4" t="n"/>
+      <c r="I59" s="4" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>TC-812</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>Processor cannot list users</t>
         </is>
@@ -2256,23 +2182,23 @@
           <t>403, FORBIDDEN</t>
         </is>
       </c>
-      <c r="F60" s="3" t="n"/>
-      <c r="G60" s="3" t="n"/>
-      <c r="H60" s="3" t="n"/>
-      <c r="I60" s="3" t="n"/>
+      <c r="F60" s="4" t="n"/>
+      <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="n"/>
+      <c r="I60" s="4" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t>TC-813</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>Processor cannot set roles</t>
         </is>
@@ -2287,23 +2213,23 @@
           <t>403, FORBIDDEN</t>
         </is>
       </c>
-      <c r="F61" s="3" t="n"/>
-      <c r="G61" s="3" t="n"/>
-      <c r="H61" s="3" t="n"/>
-      <c r="I61" s="3" t="n"/>
+      <c r="F61" s="4" t="n"/>
+      <c r="G61" s="4" t="n"/>
+      <c r="H61" s="4" t="n"/>
+      <c r="I61" s="4" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>TC-814</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Processor cannot delete roles</t>
         </is>
@@ -2318,23 +2244,23 @@
           <t>403, FORBIDDEN</t>
         </is>
       </c>
-      <c r="F62" s="3" t="n"/>
-      <c r="G62" s="3" t="n"/>
-      <c r="H62" s="3" t="n"/>
-      <c r="I62" s="3" t="n"/>
+      <c r="F62" s="4" t="n"/>
+      <c r="G62" s="4" t="n"/>
+      <c r="H62" s="4" t="n"/>
+      <c r="I62" s="4" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="inlineStr">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>TC-815</t>
         </is>
       </c>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>Unauthenticated access</t>
         </is>
@@ -2349,23 +2275,23 @@
           <t>401, UNAUTHORIZED</t>
         </is>
       </c>
-      <c r="F63" s="3" t="n"/>
-      <c r="G63" s="3" t="n"/>
-      <c r="H63" s="3" t="n"/>
-      <c r="I63" s="3" t="n"/>
+      <c r="F63" s="4" t="n"/>
+      <c r="G63" s="4" t="n"/>
+      <c r="H63" s="4" t="n"/>
+      <c r="I63" s="4" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="inlineStr">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>TC-816</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>ROLE_ASSIGNED audit log</t>
         </is>
@@ -2380,23 +2306,23 @@
           <t>Audit entry with actor, target user, and roles</t>
         </is>
       </c>
-      <c r="F64" s="3" t="n"/>
-      <c r="G64" s="3" t="n"/>
-      <c r="H64" s="3" t="n"/>
-      <c r="I64" s="3" t="n"/>
+      <c r="F64" s="4" t="n"/>
+      <c r="G64" s="4" t="n"/>
+      <c r="H64" s="4" t="n"/>
+      <c r="I64" s="4" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="inlineStr">
+      <c r="A65" s="4" t="inlineStr">
         <is>
           <t>TC-817</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr">
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>ROLE_REMOVED audit log</t>
         </is>
@@ -2411,61 +2337,61 @@
           <t>Audit entry with actor and target user</t>
         </is>
       </c>
-      <c r="F65" s="3" t="n"/>
-      <c r="G65" s="3" t="n"/>
-      <c r="H65" s="3" t="n"/>
-      <c r="I65" s="3" t="n"/>
+      <c r="F65" s="4" t="n"/>
+      <c r="G65" s="4" t="n"/>
+      <c r="H65" s="4" t="n"/>
+      <c r="I65" s="4" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>TC-818</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t>DB roles override groups</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Assign ["manager"] to qa-processor via PUT, then login</t>
+          <t>Assign ["manager"] to qa-processor via PUT, then login as qa-processor</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>JWT roles is ["manager"], not ["processor"]</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="n"/>
-      <c r="G66" s="3" t="n"/>
-      <c r="H66" s="3" t="n"/>
-      <c r="I66" s="3" t="n"/>
+          <t>JWT roles is ["manager"], not ["processor"] from OS groups</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="n"/>
+      <c r="G66" s="4" t="n"/>
+      <c r="H66" s="4" t="n"/>
+      <c r="I66" s="4" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="inlineStr">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t>TC-819</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>12.8 User Role Mgmt</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t>Fallback to group roles</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>DELETE user roles, then login as qa-processor</t>
+          <t>DELETE /users/qa-processor/roles, then login as qa-processor</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
@@ -2473,1908 +2399,1970 @@
           <t>JWT roles falls back to OS group mapping (["processor"])</t>
         </is>
       </c>
-      <c r="F67" s="3" t="n"/>
-      <c r="G67" s="3" t="n"/>
-      <c r="H67" s="3" t="n"/>
-      <c r="I67" s="3" t="n"/>
+      <c r="F67" s="4" t="n"/>
+      <c r="G67" s="4" t="n"/>
+      <c r="H67" s="4" t="n"/>
+      <c r="I67" s="4" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="6" t="inlineStr">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>§12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="B68" s="6" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C68" s="7" t="n"/>
-      <c r="D68" s="7" t="n"/>
-      <c r="E68" s="7" t="n"/>
-      <c r="F68" s="7" t="n"/>
-      <c r="G68" s="7" t="n"/>
-      <c r="H68" s="7" t="n"/>
-      <c r="I68" s="7" t="n"/>
+      <c r="C68" s="3" t="n"/>
+      <c r="D68" s="3" t="n"/>
+      <c r="E68" s="3" t="n"/>
+      <c r="F68" s="3" t="n"/>
+      <c r="G68" s="3" t="n"/>
+      <c r="H68" s="3" t="n"/>
+      <c r="I68" s="3" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="8" t="inlineStr">
+      <c r="A69" s="4" t="inlineStr">
         <is>
           <t>TC-901</t>
         </is>
       </c>
-      <c r="B69" s="8" t="inlineStr">
+      <c r="B69" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C69" s="8" t="inlineStr">
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>Create group</t>
         </is>
       </c>
-      <c r="D69" s="8" t="inlineStr">
+      <c r="D69" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-groups with {"name": "ecube-testers"}</t>
         </is>
       </c>
-      <c r="E69" s="8" t="inlineStr">
+      <c r="E69" s="4" t="inlineStr">
         <is>
           <t>201, returns name, gid, members</t>
         </is>
       </c>
-      <c r="F69" s="8" t="n"/>
-      <c r="G69" s="8" t="n"/>
-      <c r="H69" s="8" t="n"/>
-      <c r="I69" s="8" t="n"/>
+      <c r="F69" s="4" t="n"/>
+      <c r="G69" s="4" t="n"/>
+      <c r="H69" s="4" t="n"/>
+      <c r="I69" s="4" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="inlineStr">
+      <c r="A70" s="4" t="inlineStr">
         <is>
           <t>TC-902</t>
         </is>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B70" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C70" s="8" t="inlineStr">
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t>Create group without prefix</t>
         </is>
       </c>
-      <c r="D70" s="8" t="inlineStr">
+      <c r="D70" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-groups with {"name": "testers"}</t>
         </is>
       </c>
-      <c r="E70" s="8" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>422, group name must start with ecube-</t>
         </is>
       </c>
-      <c r="F70" s="8" t="n"/>
-      <c r="G70" s="8" t="n"/>
-      <c r="H70" s="8" t="n"/>
-      <c r="I70" s="8" t="n"/>
+      <c r="F70" s="4" t="n"/>
+      <c r="G70" s="4" t="n"/>
+      <c r="H70" s="4" t="n"/>
+      <c r="I70" s="4" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="inlineStr">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>TC-903</t>
         </is>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C71" s="8" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>List groups</t>
         </is>
       </c>
-      <c r="D71" s="8" t="inlineStr">
+      <c r="D71" s="4" t="inlineStr">
         <is>
           <t>GET /admin/os-groups</t>
         </is>
       </c>
-      <c r="E71" s="8" t="inlineStr">
+      <c r="E71" s="4" t="inlineStr">
         <is>
           <t>200, only ecube-* groups listed</t>
         </is>
       </c>
-      <c r="F71" s="8" t="n"/>
-      <c r="G71" s="8" t="n"/>
-      <c r="H71" s="8" t="n"/>
-      <c r="I71" s="8" t="n"/>
+      <c r="F71" s="4" t="n"/>
+      <c r="G71" s="4" t="n"/>
+      <c r="H71" s="4" t="n"/>
+      <c r="I71" s="4" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>TC-904</t>
         </is>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C72" s="8" t="inlineStr">
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t>Delete group</t>
         </is>
       </c>
-      <c r="D72" s="8" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr">
         <is>
           <t>DELETE /admin/os-groups/ecube-testers</t>
         </is>
       </c>
-      <c r="E72" s="8" t="inlineStr">
+      <c r="E72" s="4" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="F72" s="8" t="n"/>
-      <c r="G72" s="8" t="n"/>
-      <c r="H72" s="8" t="n"/>
-      <c r="I72" s="8" t="n"/>
+      <c r="F72" s="4" t="n"/>
+      <c r="G72" s="4" t="n"/>
+      <c r="H72" s="4" t="n"/>
+      <c r="I72" s="4" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="inlineStr">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>TC-905</t>
         </is>
       </c>
-      <c r="B73" s="8" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C73" s="8" t="inlineStr">
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>Delete group without prefix</t>
         </is>
       </c>
-      <c r="D73" s="8" t="inlineStr">
+      <c r="D73" s="4" t="inlineStr">
         <is>
           <t>DELETE /admin/os-groups/somegroup</t>
         </is>
       </c>
-      <c r="E73" s="8" t="inlineStr">
+      <c r="E73" s="4" t="inlineStr">
         <is>
           <t>422, group name must start with ecube-</t>
         </is>
       </c>
-      <c r="F73" s="8" t="n"/>
-      <c r="G73" s="8" t="n"/>
-      <c r="H73" s="8" t="n"/>
-      <c r="I73" s="8" t="n"/>
+      <c r="F73" s="4" t="n"/>
+      <c r="G73" s="4" t="n"/>
+      <c r="H73" s="4" t="n"/>
+      <c r="I73" s="4" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>TC-906</t>
         </is>
       </c>
-      <c r="B74" s="8" t="inlineStr">
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C74" s="8" t="inlineStr">
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>Create user</t>
         </is>
       </c>
-      <c r="D74" s="8" t="inlineStr">
+      <c r="D74" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-users with username, password, groups, roles</t>
         </is>
       </c>
-      <c r="E74" s="8" t="inlineStr">
+      <c r="E74" s="4" t="inlineStr">
         <is>
           <t>201, returns username, uid, gid, home, shell, groups</t>
         </is>
       </c>
-      <c r="F74" s="8" t="n"/>
-      <c r="G74" s="8" t="n"/>
-      <c r="H74" s="8" t="n"/>
-      <c r="I74" s="8" t="n"/>
+      <c r="F74" s="4" t="n"/>
+      <c r="G74" s="4" t="n"/>
+      <c r="H74" s="4" t="n"/>
+      <c r="I74" s="4" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="8" t="inlineStr">
+      <c r="A75" s="4" t="inlineStr">
         <is>
           <t>TC-907</t>
         </is>
       </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B75" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C75" s="8" t="inlineStr">
+      <c r="C75" s="4" t="inlineStr">
         <is>
           <t>Create user — duplicate</t>
         </is>
       </c>
-      <c r="D75" s="8" t="inlineStr">
+      <c r="D75" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-users with existing username</t>
         </is>
       </c>
-      <c r="E75" s="8" t="inlineStr">
+      <c r="E75" s="4" t="inlineStr">
         <is>
           <t>409, Conflict</t>
         </is>
       </c>
-      <c r="F75" s="8" t="n"/>
-      <c r="G75" s="8" t="n"/>
-      <c r="H75" s="8" t="n"/>
-      <c r="I75" s="8" t="n"/>
+      <c r="F75" s="4" t="n"/>
+      <c r="G75" s="4" t="n"/>
+      <c r="H75" s="4" t="n"/>
+      <c r="I75" s="4" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="8" t="inlineStr">
+      <c r="A76" s="4" t="inlineStr">
         <is>
           <t>TC-908</t>
         </is>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B76" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C76" s="8" t="inlineStr">
+      <c r="C76" s="4" t="inlineStr">
         <is>
           <t>Create user — reserved name</t>
         </is>
       </c>
-      <c r="D76" s="8" t="inlineStr">
+      <c r="D76" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-users with {"username": "root", ...}</t>
         </is>
       </c>
-      <c r="E76" s="8" t="inlineStr">
+      <c r="E76" s="4" t="inlineStr">
         <is>
           <t>422, reserved username</t>
         </is>
       </c>
-      <c r="F76" s="8" t="n"/>
-      <c r="G76" s="8" t="n"/>
-      <c r="H76" s="8" t="n"/>
-      <c r="I76" s="8" t="n"/>
+      <c r="F76" s="4" t="n"/>
+      <c r="G76" s="4" t="n"/>
+      <c r="H76" s="4" t="n"/>
+      <c r="I76" s="4" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="8" t="inlineStr">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>TC-909</t>
         </is>
       </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="B77" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C77" s="8" t="inlineStr">
+      <c r="C77" s="4" t="inlineStr">
         <is>
           <t>Create user — empty password</t>
         </is>
       </c>
-      <c r="D77" s="8" t="inlineStr">
+      <c r="D77" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-users with {"password": "", ...}</t>
         </is>
       </c>
-      <c r="E77" s="8" t="inlineStr">
+      <c r="E77" s="4" t="inlineStr">
         <is>
           <t>422</t>
         </is>
       </c>
-      <c r="F77" s="8" t="n"/>
-      <c r="G77" s="8" t="n"/>
-      <c r="H77" s="8" t="n"/>
-      <c r="I77" s="8" t="n"/>
+      <c r="F77" s="4" t="n"/>
+      <c r="G77" s="4" t="n"/>
+      <c r="H77" s="4" t="n"/>
+      <c r="I77" s="4" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="inlineStr">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <t>TC-910</t>
         </is>
       </c>
-      <c r="B78" s="8" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C78" s="8" t="inlineStr">
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>Create user — password with newline</t>
         </is>
       </c>
-      <c r="D78" s="8" t="inlineStr">
+      <c r="D78" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-users with password containing \n</t>
         </is>
       </c>
-      <c r="E78" s="8" t="inlineStr">
+      <c r="E78" s="4" t="inlineStr">
         <is>
           <t>422, unsafe characters</t>
         </is>
       </c>
-      <c r="F78" s="8" t="n"/>
-      <c r="G78" s="8" t="n"/>
-      <c r="H78" s="8" t="n"/>
-      <c r="I78" s="8" t="n"/>
+      <c r="F78" s="4" t="n"/>
+      <c r="G78" s="4" t="n"/>
+      <c r="H78" s="4" t="n"/>
+      <c r="I78" s="4" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="inlineStr">
+      <c r="A79" s="4" t="inlineStr">
         <is>
           <t>TC-911</t>
         </is>
       </c>
-      <c r="B79" s="8" t="inlineStr">
+      <c r="B79" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C79" s="8" t="inlineStr">
+      <c r="C79" s="4" t="inlineStr">
         <is>
           <t>Create user — password with colon</t>
         </is>
       </c>
-      <c r="D79" s="8" t="inlineStr">
+      <c r="D79" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-users with password containing :</t>
         </is>
       </c>
-      <c r="E79" s="8" t="inlineStr">
+      <c r="E79" s="4" t="inlineStr">
         <is>
           <t>422, unsafe characters</t>
         </is>
       </c>
-      <c r="F79" s="8" t="n"/>
-      <c r="G79" s="8" t="n"/>
-      <c r="H79" s="8" t="n"/>
-      <c r="I79" s="8" t="n"/>
+      <c r="F79" s="4" t="n"/>
+      <c r="G79" s="4" t="n"/>
+      <c r="H79" s="4" t="n"/>
+      <c r="I79" s="4" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="inlineStr">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>TC-912</t>
         </is>
       </c>
-      <c r="B80" s="8" t="inlineStr">
+      <c r="B80" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C80" s="8" t="inlineStr">
+      <c r="C80" s="4" t="inlineStr">
         <is>
           <t>Create user — invalid group</t>
         </is>
       </c>
-      <c r="D80" s="8" t="inlineStr">
+      <c r="D80" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-users with non-existent group in groups list</t>
         </is>
       </c>
-      <c r="E80" s="8" t="inlineStr">
+      <c r="E80" s="4" t="inlineStr">
         <is>
           <t>422, group does not exist</t>
         </is>
       </c>
-      <c r="F80" s="8" t="n"/>
-      <c r="G80" s="8" t="n"/>
-      <c r="H80" s="8" t="n"/>
-      <c r="I80" s="8" t="n"/>
+      <c r="F80" s="4" t="n"/>
+      <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="n"/>
+      <c r="I80" s="4" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="8" t="inlineStr">
+      <c r="A81" s="4" t="inlineStr">
         <is>
           <t>TC-913</t>
         </is>
       </c>
-      <c r="B81" s="8" t="inlineStr">
+      <c r="B81" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C81" s="8" t="inlineStr">
+      <c r="C81" s="4" t="inlineStr">
         <is>
           <t>Create user — no ecube-* group</t>
         </is>
       </c>
-      <c r="D81" s="8" t="inlineStr">
+      <c r="D81" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-users with no groups or only non-ecube-* groups</t>
         </is>
       </c>
-      <c r="E81" s="8" t="inlineStr">
+      <c r="E81" s="4" t="inlineStr">
         <is>
           <t>422, at least one ecube-* group required</t>
         </is>
       </c>
-      <c r="F81" s="8" t="n"/>
-      <c r="G81" s="8" t="n"/>
-      <c r="H81" s="8" t="n"/>
-      <c r="I81" s="8" t="n"/>
+      <c r="F81" s="4" t="n"/>
+      <c r="G81" s="4" t="n"/>
+      <c r="H81" s="4" t="n"/>
+      <c r="I81" s="4" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="inlineStr">
+      <c r="A82" s="4" t="inlineStr">
         <is>
           <t>TC-914</t>
         </is>
       </c>
-      <c r="B82" s="8" t="inlineStr">
+      <c r="B82" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C82" s="8" t="inlineStr">
+      <c r="C82" s="4" t="inlineStr">
         <is>
           <t>List users</t>
         </is>
       </c>
-      <c r="D82" s="8" t="inlineStr">
+      <c r="D82" s="4" t="inlineStr">
         <is>
           <t>GET /admin/os-users</t>
         </is>
       </c>
-      <c r="E82" s="8" t="inlineStr">
+      <c r="E82" s="4" t="inlineStr">
         <is>
           <t>200, only users in ecube-* groups listed</t>
         </is>
       </c>
-      <c r="F82" s="8" t="n"/>
-      <c r="G82" s="8" t="n"/>
-      <c r="H82" s="8" t="n"/>
-      <c r="I82" s="8" t="n"/>
+      <c r="F82" s="4" t="n"/>
+      <c r="G82" s="4" t="n"/>
+      <c r="H82" s="4" t="n"/>
+      <c r="I82" s="4" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="8" t="inlineStr">
+      <c r="A83" s="4" t="inlineStr">
         <is>
           <t>TC-915</t>
         </is>
       </c>
-      <c r="B83" s="8" t="inlineStr">
+      <c r="B83" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C83" s="8" t="inlineStr">
+      <c r="C83" s="4" t="inlineStr">
         <is>
           <t>Reset password</t>
         </is>
       </c>
-      <c r="D83" s="8" t="inlineStr">
+      <c r="D83" s="4" t="inlineStr">
         <is>
           <t>PUT /admin/os-users/{username}/password with {"password": "NewPass!"}</t>
         </is>
       </c>
-      <c r="E83" s="8" t="inlineStr">
+      <c r="E83" s="4" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="F83" s="8" t="n"/>
-      <c r="G83" s="8" t="n"/>
-      <c r="H83" s="8" t="n"/>
-      <c r="I83" s="8" t="n"/>
+      <c r="F83" s="4" t="n"/>
+      <c r="G83" s="4" t="n"/>
+      <c r="H83" s="4" t="n"/>
+      <c r="I83" s="4" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="inlineStr">
+      <c r="A84" s="4" t="inlineStr">
         <is>
           <t>TC-916</t>
         </is>
       </c>
-      <c r="B84" s="8" t="inlineStr">
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C84" s="8" t="inlineStr">
+      <c r="C84" s="4" t="inlineStr">
         <is>
           <t>Reset password — non-ECUBE user</t>
         </is>
       </c>
-      <c r="D84" s="8" t="inlineStr">
+      <c r="D84" s="4" t="inlineStr">
         <is>
           <t>PUT /admin/os-users/postgres/password</t>
         </is>
       </c>
-      <c r="E84" s="8" t="inlineStr">
+      <c r="E84" s="4" t="inlineStr">
         <is>
           <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
-      <c r="F84" s="8" t="n"/>
-      <c r="G84" s="8" t="n"/>
-      <c r="H84" s="8" t="n"/>
-      <c r="I84" s="8" t="n"/>
+      <c r="F84" s="4" t="n"/>
+      <c r="G84" s="4" t="n"/>
+      <c r="H84" s="4" t="n"/>
+      <c r="I84" s="4" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="8" t="inlineStr">
+      <c r="A85" s="4" t="inlineStr">
         <is>
           <t>TC-917</t>
         </is>
       </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="B85" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C85" s="8" t="inlineStr">
+      <c r="C85" s="4" t="inlineStr">
         <is>
           <t>Replace groups</t>
         </is>
       </c>
-      <c r="D85" s="8" t="inlineStr">
+      <c r="D85" s="4" t="inlineStr">
         <is>
           <t>PUT /admin/os-users/{username}/groups with {"groups": ["ecube-admins"]}</t>
         </is>
       </c>
-      <c r="E85" s="8" t="inlineStr">
+      <c r="E85" s="4" t="inlineStr">
         <is>
           <t>200, updated group list; non-ecube-* groups preserved</t>
         </is>
       </c>
-      <c r="F85" s="8" t="n"/>
-      <c r="G85" s="8" t="n"/>
-      <c r="H85" s="8" t="n"/>
-      <c r="I85" s="8" t="n"/>
+      <c r="F85" s="4" t="n"/>
+      <c r="G85" s="4" t="n"/>
+      <c r="H85" s="4" t="n"/>
+      <c r="I85" s="4" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="8" t="inlineStr">
+      <c r="A86" s="4" t="inlineStr">
         <is>
           <t>TC-918</t>
         </is>
       </c>
-      <c r="B86" s="8" t="inlineStr">
+      <c r="B86" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C86" s="8" t="inlineStr">
+      <c r="C86" s="4" t="inlineStr">
         <is>
           <t>Replace groups — empty list</t>
         </is>
       </c>
-      <c r="D86" s="8" t="inlineStr">
+      <c r="D86" s="4" t="inlineStr">
         <is>
           <t>PUT /admin/os-users/{username}/groups with {"groups": []}</t>
         </is>
       </c>
-      <c r="E86" s="8" t="inlineStr">
+      <c r="E86" s="4" t="inlineStr">
         <is>
           <t>422, at least one ecube-* group required</t>
         </is>
       </c>
+      <c r="F86" s="4" t="n"/>
+      <c r="G86" s="4" t="n"/>
+      <c r="H86" s="4" t="n"/>
+      <c r="I86" s="4" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="inlineStr">
+      <c r="A87" s="4" t="inlineStr">
         <is>
           <t>TC-919</t>
         </is>
       </c>
-      <c r="B87" s="8" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C87" s="8" t="inlineStr">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>Replace groups — non-ecube name</t>
         </is>
       </c>
-      <c r="D87" s="8" t="inlineStr">
+      <c r="D87" s="4" t="inlineStr">
         <is>
           <t>PUT /admin/os-users/{username}/groups with {"groups": ["docker"]}</t>
         </is>
       </c>
-      <c r="E87" s="8" t="inlineStr">
+      <c r="E87" s="4" t="inlineStr">
         <is>
           <t>422, group does not start with ecube-</t>
         </is>
       </c>
+      <c r="F87" s="4" t="n"/>
+      <c r="G87" s="4" t="n"/>
+      <c r="H87" s="4" t="n"/>
+      <c r="I87" s="4" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="8" t="inlineStr">
+      <c r="A88" s="4" t="inlineStr">
         <is>
           <t>TC-920</t>
         </is>
       </c>
-      <c r="B88" s="8" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C88" s="8" t="inlineStr">
+      <c r="C88" s="4" t="inlineStr">
         <is>
           <t>Append groups</t>
         </is>
       </c>
-      <c r="D88" s="8" t="inlineStr">
+      <c r="D88" s="4" t="inlineStr">
         <is>
           <t>POST /admin/os-users/{username}/groups with {"groups": ["ecube-managers"]}</t>
         </is>
       </c>
-      <c r="E88" s="8" t="inlineStr">
+      <c r="E88" s="4" t="inlineStr">
         <is>
           <t>200, updated group list</t>
         </is>
       </c>
-      <c r="F88" s="8" t="n"/>
-      <c r="G88" s="8" t="n"/>
-      <c r="H88" s="8" t="n"/>
-      <c r="I88" s="8" t="n"/>
+      <c r="F88" s="4" t="n"/>
+      <c r="G88" s="4" t="n"/>
+      <c r="H88" s="4" t="n"/>
+      <c r="I88" s="4" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="8" t="inlineStr">
+      <c r="A89" s="4" t="inlineStr">
         <is>
           <t>TC-921</t>
         </is>
       </c>
-      <c r="B89" s="8" t="inlineStr">
+      <c r="B89" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C89" s="8" t="inlineStr">
+      <c r="C89" s="4" t="inlineStr">
         <is>
           <t>Modify groups — non-ECUBE user</t>
         </is>
       </c>
-      <c r="D89" s="8" t="inlineStr">
+      <c r="D89" s="4" t="inlineStr">
         <is>
           <t>PUT /admin/os-users/www-data/groups</t>
         </is>
       </c>
-      <c r="E89" s="8" t="inlineStr">
+      <c r="E89" s="4" t="inlineStr">
         <is>
           <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
-      <c r="F89" s="8" t="n"/>
-      <c r="G89" s="8" t="n"/>
-      <c r="H89" s="8" t="n"/>
-      <c r="I89" s="8" t="n"/>
+      <c r="F89" s="4" t="n"/>
+      <c r="G89" s="4" t="n"/>
+      <c r="H89" s="4" t="n"/>
+      <c r="I89" s="4" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="inlineStr">
+      <c r="A90" s="4" t="inlineStr">
         <is>
           <t>TC-922</t>
         </is>
       </c>
-      <c r="B90" s="8" t="inlineStr">
+      <c r="B90" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C90" s="8" t="inlineStr">
+      <c r="C90" s="4" t="inlineStr">
         <is>
           <t>Delete user</t>
         </is>
       </c>
-      <c r="D90" s="8" t="inlineStr">
+      <c r="D90" s="4" t="inlineStr">
         <is>
           <t>DELETE /admin/os-users/{username}</t>
         </is>
       </c>
-      <c r="E90" s="8" t="inlineStr">
+      <c r="E90" s="4" t="inlineStr">
         <is>
           <t>200, user and DB roles removed</t>
         </is>
       </c>
-      <c r="F90" s="8" t="n"/>
-      <c r="G90" s="8" t="n"/>
-      <c r="H90" s="8" t="n"/>
-      <c r="I90" s="8" t="n"/>
+      <c r="F90" s="4" t="n"/>
+      <c r="G90" s="4" t="n"/>
+      <c r="H90" s="4" t="n"/>
+      <c r="I90" s="4" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="8" t="inlineStr">
+      <c r="A91" s="4" t="inlineStr">
         <is>
           <t>TC-923</t>
         </is>
       </c>
-      <c r="B91" s="8" t="inlineStr">
+      <c r="B91" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C91" s="8" t="inlineStr">
+      <c r="C91" s="4" t="inlineStr">
         <is>
           <t>Delete user — non-ECUBE user</t>
         </is>
       </c>
-      <c r="D91" s="8" t="inlineStr">
+      <c r="D91" s="4" t="inlineStr">
         <is>
           <t>DELETE /admin/os-users/daemon</t>
         </is>
       </c>
-      <c r="E91" s="8" t="inlineStr">
+      <c r="E91" s="4" t="inlineStr">
         <is>
           <t>422, user is not ECUBE-managed</t>
         </is>
       </c>
-      <c r="F91" s="8" t="n"/>
-      <c r="G91" s="8" t="n"/>
-      <c r="H91" s="8" t="n"/>
-      <c r="I91" s="8" t="n"/>
+      <c r="F91" s="4" t="n"/>
+      <c r="G91" s="4" t="n"/>
+      <c r="H91" s="4" t="n"/>
+      <c r="I91" s="4" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="8" t="inlineStr">
+      <c r="A92" s="4" t="inlineStr">
         <is>
           <t>TC-924</t>
         </is>
       </c>
-      <c r="B92" s="8" t="inlineStr">
+      <c r="B92" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C92" s="8" t="inlineStr">
+      <c r="C92" s="4" t="inlineStr">
         <is>
           <t>Delete user — not found</t>
         </is>
       </c>
-      <c r="D92" s="8" t="inlineStr">
+      <c r="D92" s="4" t="inlineStr">
         <is>
           <t>DELETE /admin/os-users/nonexistent</t>
         </is>
       </c>
-      <c r="E92" s="8" t="inlineStr">
+      <c r="E92" s="4" t="inlineStr">
         <is>
           <t>404</t>
         </is>
       </c>
-      <c r="F92" s="8" t="n"/>
-      <c r="G92" s="8" t="n"/>
-      <c r="H92" s="8" t="n"/>
-      <c r="I92" s="8" t="n"/>
+      <c r="F92" s="4" t="n"/>
+      <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="n"/>
+      <c r="I92" s="4" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="inlineStr">
+      <c r="A93" s="4" t="inlineStr">
         <is>
           <t>TC-925</t>
         </is>
       </c>
-      <c r="B93" s="8" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C93" s="8" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>Processor cannot access OS endpoints</t>
         </is>
       </c>
-      <c r="D93" s="8" t="inlineStr">
+      <c r="D93" s="4" t="inlineStr">
         <is>
           <t>GET /admin/os-users with processor token</t>
         </is>
       </c>
-      <c r="E93" s="8" t="inlineStr">
+      <c r="E93" s="4" t="inlineStr">
         <is>
           <t>403, FORBIDDEN</t>
         </is>
       </c>
-      <c r="F93" s="8" t="n"/>
-      <c r="G93" s="8" t="n"/>
-      <c r="H93" s="8" t="n"/>
-      <c r="I93" s="8" t="n"/>
+      <c r="F93" s="4" t="n"/>
+      <c r="G93" s="4" t="n"/>
+      <c r="H93" s="4" t="n"/>
+      <c r="I93" s="4" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="inlineStr">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>TC-926</t>
         </is>
       </c>
-      <c r="B94" s="8" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C94" s="8" t="inlineStr">
+      <c r="C94" s="4" t="inlineStr">
         <is>
           <t>Non-local mode returns 404</t>
         </is>
       </c>
-      <c r="D94" s="8" t="inlineStr">
+      <c r="D94" s="4" t="inlineStr">
         <is>
           <t>All /admin/os-* endpoints when role_resolver != "local"</t>
         </is>
       </c>
-      <c r="E94" s="8" t="inlineStr">
+      <c r="E94" s="4" t="inlineStr">
         <is>
           <t>404, Not Found</t>
         </is>
       </c>
-      <c r="F94" s="8" t="n"/>
-      <c r="G94" s="8" t="n"/>
-      <c r="H94" s="8" t="n"/>
-      <c r="I94" s="8" t="n"/>
+      <c r="F94" s="4" t="n"/>
+      <c r="G94" s="4" t="n"/>
+      <c r="H94" s="4" t="n"/>
+      <c r="I94" s="4" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="8" t="inlineStr">
+      <c r="A95" s="4" t="inlineStr">
         <is>
           <t>TC-927</t>
         </is>
       </c>
-      <c r="B95" s="8" t="inlineStr">
+      <c r="B95" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C95" s="8" t="inlineStr">
+      <c r="C95" s="4" t="inlineStr">
         <is>
           <t>OS_USER_CREATED audit log</t>
         </is>
       </c>
-      <c r="D95" s="8" t="inlineStr">
+      <c r="D95" s="4" t="inlineStr">
         <is>
           <t>GET /audit?action=OS_USER_CREATED after creating user</t>
         </is>
       </c>
-      <c r="E95" s="8" t="inlineStr">
+      <c r="E95" s="4" t="inlineStr">
         <is>
           <t>Audit entry with actor and username</t>
         </is>
       </c>
-      <c r="F95" s="8" t="n"/>
-      <c r="G95" s="8" t="n"/>
-      <c r="H95" s="8" t="n"/>
-      <c r="I95" s="8" t="n"/>
+      <c r="F95" s="4" t="n"/>
+      <c r="G95" s="4" t="n"/>
+      <c r="H95" s="4" t="n"/>
+      <c r="I95" s="4" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="8" t="inlineStr">
+      <c r="A96" s="4" t="inlineStr">
         <is>
           <t>TC-928</t>
         </is>
       </c>
-      <c r="B96" s="8" t="inlineStr">
+      <c r="B96" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C96" s="8" t="inlineStr">
+      <c r="C96" s="4" t="inlineStr">
         <is>
           <t>OS_USER_DELETED audit log</t>
         </is>
       </c>
-      <c r="D96" s="8" t="inlineStr">
+      <c r="D96" s="4" t="inlineStr">
         <is>
           <t>GET /audit?action=OS_USER_DELETED after deleting user</t>
         </is>
       </c>
-      <c r="E96" s="8" t="inlineStr">
+      <c r="E96" s="4" t="inlineStr">
         <is>
           <t>Audit entry with actor and username</t>
         </is>
       </c>
-      <c r="F96" s="8" t="n"/>
-      <c r="G96" s="8" t="n"/>
-      <c r="H96" s="8" t="n"/>
-      <c r="I96" s="8" t="n"/>
+      <c r="F96" s="4" t="n"/>
+      <c r="G96" s="4" t="n"/>
+      <c r="H96" s="4" t="n"/>
+      <c r="I96" s="4" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="8" t="inlineStr">
+      <c r="A97" s="4" t="inlineStr">
         <is>
           <t>TC-929</t>
         </is>
       </c>
-      <c r="B97" s="8" t="inlineStr">
+      <c r="B97" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C97" s="8" t="inlineStr">
+      <c r="C97" s="4" t="inlineStr">
         <is>
           <t>OS_PASSWORD_RESET audit log</t>
         </is>
       </c>
-      <c r="D97" s="8" t="inlineStr">
+      <c r="D97" s="4" t="inlineStr">
         <is>
           <t>GET /audit?action=OS_PASSWORD_RESET after resetting password</t>
         </is>
       </c>
-      <c r="E97" s="8" t="inlineStr">
+      <c r="E97" s="4" t="inlineStr">
         <is>
           <t>Audit entry (no password in details)</t>
         </is>
       </c>
-      <c r="F97" s="8" t="n"/>
-      <c r="G97" s="8" t="n"/>
-      <c r="H97" s="8" t="n"/>
-      <c r="I97" s="8" t="n"/>
+      <c r="F97" s="4" t="n"/>
+      <c r="G97" s="4" t="n"/>
+      <c r="H97" s="4" t="n"/>
+      <c r="I97" s="4" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="8" t="inlineStr">
+      <c r="A98" s="4" t="inlineStr">
         <is>
           <t>TC-930</t>
         </is>
       </c>
-      <c r="B98" s="8" t="inlineStr">
+      <c r="B98" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C98" s="8" t="inlineStr">
+      <c r="C98" s="4" t="inlineStr">
         <is>
           <t>OS_GROUP_CREATED audit log</t>
         </is>
       </c>
-      <c r="D98" s="8" t="inlineStr">
+      <c r="D98" s="4" t="inlineStr">
         <is>
           <t>GET /audit?action=OS_GROUP_CREATED after creating group</t>
         </is>
       </c>
-      <c r="E98" s="8" t="inlineStr">
+      <c r="E98" s="4" t="inlineStr">
         <is>
           <t>Audit entry with group name</t>
         </is>
       </c>
-      <c r="F98" s="8" t="n"/>
-      <c r="G98" s="8" t="n"/>
-      <c r="H98" s="8" t="n"/>
-      <c r="I98" s="8" t="n"/>
+      <c r="F98" s="4" t="n"/>
+      <c r="G98" s="4" t="n"/>
+      <c r="H98" s="4" t="n"/>
+      <c r="I98" s="4" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="8" t="inlineStr">
+      <c r="A99" s="4" t="inlineStr">
         <is>
           <t>TC-931</t>
         </is>
       </c>
-      <c r="B99" s="8" t="inlineStr">
+      <c r="B99" s="4" t="inlineStr">
         <is>
           <t>12.9 OS User &amp; Group Mgmt</t>
         </is>
       </c>
-      <c r="C99" s="8" t="inlineStr">
+      <c r="C99" s="4" t="inlineStr">
         <is>
           <t>OS_GROUP_DELETED audit log</t>
         </is>
       </c>
-      <c r="D99" s="8" t="inlineStr">
+      <c r="D99" s="4" t="inlineStr">
         <is>
           <t>GET /audit?action=OS_GROUP_DELETED after deleting group</t>
         </is>
       </c>
-      <c r="E99" s="8" t="inlineStr">
+      <c r="E99" s="4" t="inlineStr">
         <is>
           <t>Audit entry with group name</t>
         </is>
       </c>
-      <c r="F99" s="8" t="n"/>
-      <c r="G99" s="8" t="n"/>
-      <c r="H99" s="8" t="n"/>
-      <c r="I99" s="8" t="n"/>
+      <c r="F99" s="4" t="n"/>
+      <c r="G99" s="4" t="n"/>
+      <c r="H99" s="4" t="n"/>
+      <c r="I99" s="4" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="6" t="inlineStr">
+      <c r="A100" s="2" t="inlineStr">
         <is>
           <t>§12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="B100" s="6" t="inlineStr">
+      <c r="B100" s="2" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C100" s="7" t="n"/>
-      <c r="D100" s="7" t="n"/>
-      <c r="E100" s="7" t="n"/>
-      <c r="F100" s="7" t="n"/>
-      <c r="G100" s="7" t="n"/>
-      <c r="H100" s="7" t="n"/>
-      <c r="I100" s="7" t="n"/>
+      <c r="C100" s="3" t="n"/>
+      <c r="D100" s="3" t="n"/>
+      <c r="E100" s="3" t="n"/>
+      <c r="F100" s="3" t="n"/>
+      <c r="G100" s="3" t="n"/>
+      <c r="H100" s="3" t="n"/>
+      <c r="I100" s="3" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="8" t="inlineStr">
+      <c r="A101" s="4" t="inlineStr">
         <is>
           <t>TC-1001</t>
         </is>
       </c>
-      <c r="B101" s="8" t="inlineStr">
+      <c r="B101" s="4" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C101" s="8" t="inlineStr">
+      <c r="C101" s="4" t="inlineStr">
         <is>
           <t>Status — not initialized</t>
         </is>
       </c>
-      <c r="D101" s="8" t="inlineStr">
+      <c r="D101" s="4" t="inlineStr">
         <is>
           <t>GET /setup/status on fresh database</t>
         </is>
       </c>
-      <c r="E101" s="8" t="inlineStr">
+      <c r="E101" s="4" t="inlineStr">
         <is>
           <t>200, {"initialized": false}</t>
         </is>
       </c>
-      <c r="F101" s="8" t="n"/>
-      <c r="G101" s="8" t="n"/>
-      <c r="H101" s="8" t="n"/>
-      <c r="I101" s="8" t="n"/>
+      <c r="F101" s="4" t="n"/>
+      <c r="G101" s="4" t="n"/>
+      <c r="H101" s="4" t="n"/>
+      <c r="I101" s="4" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="8" t="inlineStr">
+      <c r="A102" s="4" t="inlineStr">
         <is>
           <t>TC-1002</t>
         </is>
       </c>
-      <c r="B102" s="8" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C102" s="8" t="inlineStr">
+      <c r="C102" s="4" t="inlineStr">
         <is>
           <t>Initialize</t>
         </is>
       </c>
-      <c r="D102" s="8" t="inlineStr">
+      <c r="D102" s="4" t="inlineStr">
         <is>
           <t>POST /setup/initialize with valid username and password</t>
         </is>
       </c>
-      <c r="E102" s="8" t="inlineStr">
+      <c r="E102" s="4" t="inlineStr">
         <is>
           <t>200, returns message, username, groups_created</t>
         </is>
       </c>
-      <c r="F102" s="8" t="n"/>
-      <c r="G102" s="8" t="n"/>
-      <c r="H102" s="8" t="n"/>
-      <c r="I102" s="8" t="n"/>
+      <c r="F102" s="4" t="n"/>
+      <c r="G102" s="4" t="n"/>
+      <c r="H102" s="4" t="n"/>
+      <c r="I102" s="4" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="8" t="inlineStr">
+      <c r="A103" s="4" t="inlineStr">
         <is>
           <t>TC-1003</t>
         </is>
       </c>
-      <c r="B103" s="8" t="inlineStr">
+      <c r="B103" s="4" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C103" s="8" t="inlineStr">
+      <c r="C103" s="4" t="inlineStr">
         <is>
           <t>Status — initialized</t>
         </is>
       </c>
-      <c r="D103" s="8" t="inlineStr">
+      <c r="D103" s="4" t="inlineStr">
         <is>
           <t>GET /setup/status after initialization</t>
         </is>
       </c>
-      <c r="E103" s="8" t="inlineStr">
+      <c r="E103" s="4" t="inlineStr">
         <is>
           <t>200, {"initialized": true}</t>
         </is>
       </c>
-      <c r="F103" s="8" t="n"/>
-      <c r="G103" s="8" t="n"/>
-      <c r="H103" s="8" t="n"/>
-      <c r="I103" s="8" t="n"/>
+      <c r="F103" s="4" t="n"/>
+      <c r="G103" s="4" t="n"/>
+      <c r="H103" s="4" t="n"/>
+      <c r="I103" s="4" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="8" t="inlineStr">
+      <c r="A104" s="4" t="inlineStr">
         <is>
           <t>TC-1004</t>
         </is>
       </c>
-      <c r="B104" s="8" t="inlineStr">
+      <c r="B104" s="4" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C104" s="8" t="inlineStr">
+      <c r="C104" s="4" t="inlineStr">
         <is>
           <t>Re-initialize rejected</t>
         </is>
       </c>
-      <c r="D104" s="8" t="inlineStr">
+      <c r="D104" s="4" t="inlineStr">
         <is>
           <t>POST /setup/initialize again</t>
         </is>
       </c>
-      <c r="E104" s="8" t="inlineStr">
+      <c r="E104" s="4" t="inlineStr">
         <is>
           <t>409, Conflict</t>
         </is>
       </c>
-      <c r="F104" s="8" t="n"/>
-      <c r="G104" s="8" t="n"/>
-      <c r="H104" s="8" t="n"/>
-      <c r="I104" s="8" t="n"/>
+      <c r="F104" s="4" t="n"/>
+      <c r="G104" s="4" t="n"/>
+      <c r="H104" s="4" t="n"/>
+      <c r="I104" s="4" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="8" t="inlineStr">
+      <c r="A105" s="4" t="inlineStr">
         <is>
           <t>TC-1005</t>
         </is>
       </c>
-      <c r="B105" s="8" t="inlineStr">
+      <c r="B105" s="4" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C105" s="8" t="inlineStr">
+      <c r="C105" s="4" t="inlineStr">
         <is>
           <t>Invalid username</t>
         </is>
       </c>
-      <c r="D105" s="8" t="inlineStr">
+      <c r="D105" s="4" t="inlineStr">
         <is>
           <t>POST /setup/initialize with uppercase or special chars</t>
         </is>
       </c>
-      <c r="E105" s="8" t="inlineStr">
+      <c r="E105" s="4" t="inlineStr">
         <is>
           <t>422</t>
         </is>
       </c>
-      <c r="F105" s="8" t="n"/>
-      <c r="G105" s="8" t="n"/>
-      <c r="H105" s="8" t="n"/>
-      <c r="I105" s="8" t="n"/>
+      <c r="F105" s="4" t="n"/>
+      <c r="G105" s="4" t="n"/>
+      <c r="H105" s="4" t="n"/>
+      <c r="I105" s="4" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="8" t="inlineStr">
+      <c r="A106" s="4" t="inlineStr">
         <is>
           <t>TC-1006</t>
         </is>
       </c>
-      <c r="B106" s="8" t="inlineStr">
+      <c r="B106" s="4" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C106" s="8" t="inlineStr">
+      <c r="C106" s="4" t="inlineStr">
         <is>
           <t>Empty password</t>
         </is>
       </c>
-      <c r="D106" s="8" t="inlineStr">
+      <c r="D106" s="4" t="inlineStr">
         <is>
           <t>POST /setup/initialize with {"password": ""}</t>
         </is>
       </c>
-      <c r="E106" s="8" t="inlineStr">
+      <c r="E106" s="4" t="inlineStr">
         <is>
           <t>422</t>
         </is>
       </c>
-      <c r="F106" s="8" t="n"/>
-      <c r="G106" s="8" t="n"/>
-      <c r="H106" s="8" t="n"/>
-      <c r="I106" s="8" t="n"/>
+      <c r="F106" s="4" t="n"/>
+      <c r="G106" s="4" t="n"/>
+      <c r="H106" s="4" t="n"/>
+      <c r="I106" s="4" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="8" t="inlineStr">
+      <c r="A107" s="4" t="inlineStr">
         <is>
           <t>TC-1007</t>
         </is>
       </c>
-      <c r="B107" s="8" t="inlineStr">
+      <c r="B107" s="4" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C107" s="8" t="inlineStr">
+      <c r="C107" s="4" t="inlineStr">
         <is>
           <t>Unsafe password chars</t>
         </is>
       </c>
-      <c r="D107" s="8" t="inlineStr">
+      <c r="D107" s="4" t="inlineStr">
         <is>
           <t>POST /setup/initialize with password containing newline or colon</t>
         </is>
       </c>
-      <c r="E107" s="8" t="inlineStr">
+      <c r="E107" s="4" t="inlineStr">
         <is>
           <t>422, unsafe characters</t>
         </is>
       </c>
-      <c r="F107" s="8" t="n"/>
-      <c r="G107" s="8" t="n"/>
-      <c r="H107" s="8" t="n"/>
-      <c r="I107" s="8" t="n"/>
+      <c r="F107" s="4" t="n"/>
+      <c r="G107" s="4" t="n"/>
+      <c r="H107" s="4" t="n"/>
+      <c r="I107" s="4" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="8" t="inlineStr">
+      <c r="A108" s="4" t="inlineStr">
         <is>
           <t>TC-1008</t>
         </is>
       </c>
-      <c r="B108" s="8" t="inlineStr">
+      <c r="B108" s="4" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C108" s="8" t="inlineStr">
+      <c r="C108" s="4" t="inlineStr">
         <is>
           <t>Login as initialized admin</t>
         </is>
       </c>
-      <c r="D108" s="8" t="inlineStr">
-        <is>
-          <t>POST /auth/token with admin credentials from initialization</t>
-        </is>
-      </c>
-      <c r="E108" s="8" t="inlineStr">
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>POST /auth/token with the admin credentials from step 2</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
         <is>
           <t>200, JWT contains admin role</t>
         </is>
       </c>
-      <c r="F108" s="8" t="n"/>
-      <c r="G108" s="8" t="n"/>
-      <c r="H108" s="8" t="n"/>
-      <c r="I108" s="8" t="n"/>
+      <c r="F108" s="4" t="n"/>
+      <c r="G108" s="4" t="n"/>
+      <c r="H108" s="4" t="n"/>
+      <c r="I108" s="4" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="8" t="inlineStr">
+      <c r="A109" s="4" t="inlineStr">
         <is>
           <t>TC-1009</t>
         </is>
       </c>
-      <c r="B109" s="8" t="inlineStr">
+      <c r="B109" s="4" t="inlineStr">
         <is>
           <t>12.10 First-Run Setup</t>
         </is>
       </c>
-      <c r="C109" s="8" t="inlineStr">
+      <c r="C109" s="4" t="inlineStr">
         <is>
           <t>SYSTEM_INITIALIZED audit log</t>
         </is>
       </c>
-      <c r="D109" s="8" t="inlineStr">
+      <c r="D109" s="4" t="inlineStr">
         <is>
           <t>GET /audit?action=SYSTEM_INITIALIZED</t>
         </is>
       </c>
-      <c r="E109" s="8" t="inlineStr">
+      <c r="E109" s="4" t="inlineStr">
         <is>
           <t>Audit entry with actor</t>
         </is>
       </c>
-      <c r="F109" s="8" t="n"/>
-      <c r="G109" s="8" t="n"/>
-      <c r="H109" s="8" t="n"/>
-      <c r="I109" s="8" t="n"/>
+      <c r="F109" s="4" t="n"/>
+      <c r="G109" s="4" t="n"/>
+      <c r="H109" s="4" t="n"/>
+      <c r="I109" s="4" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="6" t="inlineStr">
+      <c r="A110" s="2" t="inlineStr">
         <is>
           <t>§12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="B110" s="6" t="inlineStr">
+      <c r="B110" s="2" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C110" s="7" t="n"/>
-      <c r="D110" s="7" t="n"/>
-      <c r="E110" s="7" t="n"/>
-      <c r="F110" s="7" t="n"/>
-      <c r="G110" s="7" t="n"/>
-      <c r="H110" s="7" t="n"/>
-      <c r="I110" s="7" t="n"/>
+      <c r="C110" s="3" t="n"/>
+      <c r="D110" s="3" t="n"/>
+      <c r="E110" s="3" t="n"/>
+      <c r="F110" s="3" t="n"/>
+      <c r="G110" s="3" t="n"/>
+      <c r="H110" s="3" t="n"/>
+      <c r="I110" s="3" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="8" t="inlineStr">
+      <c r="A111" s="4" t="inlineStr">
         <is>
           <t>TC-1101</t>
         </is>
       </c>
-      <c r="B111" s="8" t="inlineStr">
+      <c r="B111" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C111" s="8" t="inlineStr">
+      <c r="C111" s="4" t="inlineStr">
         <is>
           <t>Test connection — success</t>
         </is>
       </c>
-      <c r="D111" s="8" t="inlineStr">
+      <c r="D111" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/test-connection with valid PostgreSQL credentials</t>
         </is>
       </c>
-      <c r="E111" s="8" t="inlineStr">
+      <c r="E111" s="4" t="inlineStr">
         <is>
           <t>200, {"status": "ok", "server_version": "..."}</t>
         </is>
       </c>
-      <c r="F111" s="8" t="n"/>
-      <c r="G111" s="8" t="n"/>
-      <c r="H111" s="8" t="n"/>
-      <c r="I111" s="8" t="n"/>
+      <c r="F111" s="4" t="n"/>
+      <c r="G111" s="4" t="n"/>
+      <c r="H111" s="4" t="n"/>
+      <c r="I111" s="4" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="8" t="inlineStr">
+      <c r="A112" s="4" t="inlineStr">
         <is>
           <t>TC-1102</t>
         </is>
       </c>
-      <c r="B112" s="8" t="inlineStr">
+      <c r="B112" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C112" s="8" t="inlineStr">
+      <c r="C112" s="4" t="inlineStr">
         <is>
           <t>Test connection — bad host</t>
         </is>
       </c>
-      <c r="D112" s="8" t="inlineStr">
+      <c r="D112" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/test-connection with unreachable host</t>
         </is>
       </c>
-      <c r="E112" s="8" t="inlineStr">
+      <c r="E112" s="4" t="inlineStr">
         <is>
           <t>400, connection error</t>
         </is>
       </c>
-      <c r="F112" s="8" t="n"/>
-      <c r="G112" s="8" t="n"/>
-      <c r="H112" s="8" t="n"/>
-      <c r="I112" s="8" t="n"/>
+      <c r="F112" s="4" t="n"/>
+      <c r="G112" s="4" t="n"/>
+      <c r="H112" s="4" t="n"/>
+      <c r="I112" s="4" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="8" t="inlineStr">
+      <c r="A113" s="4" t="inlineStr">
         <is>
           <t>TC-1103</t>
         </is>
       </c>
-      <c r="B113" s="8" t="inlineStr">
+      <c r="B113" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C113" s="8" t="inlineStr">
+      <c r="C113" s="4" t="inlineStr">
         <is>
           <t>Test connection — SSRF host</t>
         </is>
       </c>
-      <c r="D113" s="8" t="inlineStr">
+      <c r="D113" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/test-connection with "host": "http://evil.com"</t>
         </is>
       </c>
-      <c r="E113" s="8" t="inlineStr">
+      <c r="E113" s="4" t="inlineStr">
         <is>
           <t>422, invalid host</t>
         </is>
       </c>
-      <c r="F113" s="8" t="n"/>
-      <c r="G113" s="8" t="n"/>
-      <c r="H113" s="8" t="n"/>
-      <c r="I113" s="8" t="n"/>
+      <c r="F113" s="4" t="n"/>
+      <c r="G113" s="4" t="n"/>
+      <c r="H113" s="4" t="n"/>
+      <c r="I113" s="4" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="8" t="inlineStr">
+      <c r="A114" s="4" t="inlineStr">
         <is>
           <t>TC-1104</t>
         </is>
       </c>
-      <c r="B114" s="8" t="inlineStr">
+      <c r="B114" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C114" s="8" t="inlineStr">
+      <c r="C114" s="4" t="inlineStr">
         <is>
           <t>Test connection — port out of range</t>
         </is>
       </c>
-      <c r="D114" s="8" t="inlineStr">
+      <c r="D114" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/test-connection with "port": 99999</t>
         </is>
       </c>
-      <c r="E114" s="8" t="inlineStr">
+      <c r="E114" s="4" t="inlineStr">
         <is>
           <t>422</t>
         </is>
       </c>
-      <c r="F114" s="8" t="n"/>
-      <c r="G114" s="8" t="n"/>
-      <c r="H114" s="8" t="n"/>
-      <c r="I114" s="8" t="n"/>
+      <c r="F114" s="4" t="n"/>
+      <c r="G114" s="4" t="n"/>
+      <c r="H114" s="4" t="n"/>
+      <c r="I114" s="4" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="8" t="inlineStr">
+      <c r="A115" s="4" t="inlineStr">
         <is>
           <t>TC-1105</t>
         </is>
       </c>
-      <c r="B115" s="8" t="inlineStr">
+      <c r="B115" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C115" s="8" t="inlineStr">
+      <c r="C115" s="4" t="inlineStr">
         <is>
           <t>Provision — success</t>
         </is>
       </c>
-      <c r="D115" s="8" t="inlineStr">
+      <c r="D115" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/provision with valid credentials</t>
         </is>
       </c>
-      <c r="E115" s="8" t="inlineStr">
+      <c r="E115" s="4" t="inlineStr">
         <is>
           <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
-      <c r="F115" s="8" t="n"/>
-      <c r="G115" s="8" t="n"/>
-      <c r="H115" s="8" t="n"/>
-      <c r="I115" s="8" t="n"/>
+      <c r="F115" s="4" t="n"/>
+      <c r="G115" s="4" t="n"/>
+      <c r="H115" s="4" t="n"/>
+      <c r="I115" s="4" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="8" t="inlineStr">
+      <c r="A116" s="4" t="inlineStr">
         <is>
           <t>TC-1106</t>
         </is>
       </c>
-      <c r="B116" s="8" t="inlineStr">
+      <c r="B116" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C116" s="8" t="inlineStr">
+      <c r="C116" s="4" t="inlineStr">
         <is>
           <t>Provision — bad admin credentials</t>
         </is>
       </c>
-      <c r="D116" s="8" t="inlineStr">
+      <c r="D116" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/provision with wrong admin password</t>
         </is>
       </c>
-      <c r="E116" s="8" t="inlineStr">
+      <c r="E116" s="4" t="inlineStr">
         <is>
           <t>400, connection error</t>
         </is>
       </c>
-      <c r="F116" s="8" t="n"/>
-      <c r="G116" s="8" t="n"/>
-      <c r="H116" s="8" t="n"/>
-      <c r="I116" s="8" t="n"/>
+      <c r="F116" s="4" t="n"/>
+      <c r="G116" s="4" t="n"/>
+      <c r="H116" s="4" t="n"/>
+      <c r="I116" s="4" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="8" t="inlineStr">
+      <c r="A117" s="4" t="inlineStr">
         <is>
           <t>TC-1107</t>
         </is>
       </c>
-      <c r="B117" s="8" t="inlineStr">
+      <c r="B117" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C117" s="8" t="inlineStr">
+      <c r="C117" s="4" t="inlineStr">
         <is>
           <t>Provision — invalid database name</t>
         </is>
       </c>
-      <c r="D117" s="8" t="inlineStr">
+      <c r="D117" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/provision with "app_database": "drop;--"</t>
         </is>
       </c>
-      <c r="E117" s="8" t="inlineStr">
+      <c r="E117" s="4" t="inlineStr">
         <is>
           <t>422, invalid identifier</t>
         </is>
       </c>
-      <c r="F117" s="8" t="n"/>
-      <c r="G117" s="8" t="n"/>
-      <c r="H117" s="8" t="n"/>
-      <c r="I117" s="8" t="n"/>
+      <c r="F117" s="4" t="n"/>
+      <c r="G117" s="4" t="n"/>
+      <c r="H117" s="4" t="n"/>
+      <c r="I117" s="4" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="8" t="inlineStr">
+      <c r="A118" s="4" t="inlineStr">
         <is>
           <t>TC-1108</t>
         </is>
       </c>
-      <c r="B118" s="8" t="inlineStr">
+      <c r="B118" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C118" s="8" t="inlineStr">
+      <c r="C118" s="4" t="inlineStr">
         <is>
           <t>Status — connected</t>
         </is>
       </c>
-      <c r="D118" s="8" t="inlineStr">
+      <c r="D118" s="4" t="inlineStr">
         <is>
           <t>GET /setup/database/status with admin token</t>
         </is>
       </c>
-      <c r="E118" s="8" t="inlineStr">
+      <c r="E118" s="4" t="inlineStr">
         <is>
           <t>200, connected: true, migration info</t>
         </is>
       </c>
-      <c r="F118" s="8" t="n"/>
-      <c r="G118" s="8" t="n"/>
-      <c r="H118" s="8" t="n"/>
-      <c r="I118" s="8" t="n"/>
+      <c r="F118" s="4" t="n"/>
+      <c r="G118" s="4" t="n"/>
+      <c r="H118" s="4" t="n"/>
+      <c r="I118" s="4" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="8" t="inlineStr">
+      <c r="A119" s="4" t="inlineStr">
         <is>
           <t>TC-1109</t>
         </is>
       </c>
-      <c r="B119" s="8" t="inlineStr">
+      <c r="B119" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C119" s="8" t="inlineStr">
+      <c r="C119" s="4" t="inlineStr">
         <is>
           <t>Status — requires auth</t>
         </is>
       </c>
-      <c r="D119" s="8" t="inlineStr">
+      <c r="D119" s="4" t="inlineStr">
         <is>
           <t>GET /setup/database/status without token</t>
         </is>
       </c>
-      <c r="E119" s="8" t="inlineStr">
+      <c r="E119" s="4" t="inlineStr">
         <is>
           <t>401</t>
         </is>
       </c>
-      <c r="F119" s="8" t="n"/>
-      <c r="G119" s="8" t="n"/>
-      <c r="H119" s="8" t="n"/>
-      <c r="I119" s="8" t="n"/>
+      <c r="F119" s="4" t="n"/>
+      <c r="G119" s="4" t="n"/>
+      <c r="H119" s="4" t="n"/>
+      <c r="I119" s="4" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="8" t="inlineStr">
+      <c r="A120" s="4" t="inlineStr">
         <is>
           <t>TC-1110</t>
         </is>
       </c>
-      <c r="B120" s="8" t="inlineStr">
+      <c r="B120" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C120" s="8" t="inlineStr">
+      <c r="C120" s="4" t="inlineStr">
         <is>
           <t>Status — requires admin</t>
         </is>
       </c>
-      <c r="D120" s="8" t="inlineStr">
+      <c r="D120" s="4" t="inlineStr">
         <is>
           <t>GET /setup/database/status with processor token</t>
         </is>
       </c>
-      <c r="E120" s="8" t="inlineStr">
+      <c r="E120" s="4" t="inlineStr">
         <is>
           <t>403</t>
         </is>
       </c>
-      <c r="F120" s="8" t="n"/>
-      <c r="G120" s="8" t="n"/>
-      <c r="H120" s="8" t="n"/>
-      <c r="I120" s="8" t="n"/>
+      <c r="F120" s="4" t="n"/>
+      <c r="G120" s="4" t="n"/>
+      <c r="H120" s="4" t="n"/>
+      <c r="I120" s="4" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="8" t="inlineStr">
+      <c r="A121" s="4" t="inlineStr">
         <is>
           <t>TC-1111</t>
         </is>
       </c>
-      <c r="B121" s="8" t="inlineStr">
+      <c r="B121" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C121" s="8" t="inlineStr">
+      <c r="C121" s="4" t="inlineStr">
         <is>
           <t>Settings update — success</t>
         </is>
       </c>
-      <c r="D121" s="8" t="inlineStr">
+      <c r="D121" s="4" t="inlineStr">
         <is>
           <t>PUT /setup/database/settings with valid partial update</t>
         </is>
       </c>
-      <c r="E121" s="8" t="inlineStr">
+      <c r="E121" s="4" t="inlineStr">
         <is>
           <t>200, {"status": "updated", ...}</t>
         </is>
       </c>
-      <c r="F121" s="8" t="n"/>
-      <c r="G121" s="8" t="n"/>
-      <c r="H121" s="8" t="n"/>
-      <c r="I121" s="8" t="n"/>
+      <c r="F121" s="4" t="n"/>
+      <c r="G121" s="4" t="n"/>
+      <c r="H121" s="4" t="n"/>
+      <c r="I121" s="4" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="8" t="inlineStr">
+      <c r="A122" s="4" t="inlineStr">
         <is>
           <t>TC-1112</t>
         </is>
       </c>
-      <c r="B122" s="8" t="inlineStr">
+      <c r="B122" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C122" s="8" t="inlineStr">
+      <c r="C122" s="4" t="inlineStr">
         <is>
           <t>Settings update — bad connection</t>
         </is>
       </c>
-      <c r="D122" s="8" t="inlineStr">
+      <c r="D122" s="4" t="inlineStr">
         <is>
           <t>PUT /setup/database/settings with unreachable host</t>
         </is>
       </c>
-      <c r="E122" s="8" t="inlineStr">
+      <c r="E122" s="4" t="inlineStr">
         <is>
           <t>400, connection test failed</t>
         </is>
       </c>
-      <c r="F122" s="8" t="n"/>
-      <c r="G122" s="8" t="n"/>
-      <c r="H122" s="8" t="n"/>
-      <c r="I122" s="8" t="n"/>
+      <c r="F122" s="4" t="n"/>
+      <c r="G122" s="4" t="n"/>
+      <c r="H122" s="4" t="n"/>
+      <c r="I122" s="4" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="8" t="inlineStr">
+      <c r="A123" s="4" t="inlineStr">
         <is>
           <t>TC-1113</t>
         </is>
       </c>
-      <c r="B123" s="8" t="inlineStr">
+      <c r="B123" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C123" s="8" t="inlineStr">
+      <c r="C123" s="4" t="inlineStr">
         <is>
           <t>Settings update — empty body</t>
         </is>
       </c>
-      <c r="D123" s="8" t="inlineStr">
+      <c r="D123" s="4" t="inlineStr">
         <is>
           <t>PUT /setup/database/settings with {}</t>
         </is>
       </c>
-      <c r="E123" s="8" t="inlineStr">
+      <c r="E123" s="4" t="inlineStr">
         <is>
           <t>422, at least one field required</t>
         </is>
       </c>
-      <c r="F123" s="8" t="n"/>
-      <c r="G123" s="8" t="n"/>
-      <c r="H123" s="8" t="n"/>
-      <c r="I123" s="8" t="n"/>
+      <c r="F123" s="4" t="n"/>
+      <c r="G123" s="4" t="n"/>
+      <c r="H123" s="4" t="n"/>
+      <c r="I123" s="4" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="8" t="inlineStr">
+      <c r="A124" s="4" t="inlineStr">
         <is>
           <t>TC-1114</t>
         </is>
       </c>
-      <c r="B124" s="8" t="inlineStr">
+      <c r="B124" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C124" s="8" t="inlineStr">
+      <c r="C124" s="4" t="inlineStr">
         <is>
           <t>Settings update — requires admin</t>
         </is>
       </c>
-      <c r="D124" s="8" t="inlineStr">
+      <c r="D124" s="4" t="inlineStr">
         <is>
           <t>PUT /setup/database/settings with processor token</t>
         </is>
       </c>
-      <c r="E124" s="8" t="inlineStr">
+      <c r="E124" s="4" t="inlineStr">
         <is>
           <t>403</t>
         </is>
       </c>
-      <c r="F124" s="8" t="n"/>
-      <c r="G124" s="8" t="n"/>
-      <c r="H124" s="8" t="n"/>
-      <c r="I124" s="8" t="n"/>
+      <c r="F124" s="4" t="n"/>
+      <c r="G124" s="4" t="n"/>
+      <c r="H124" s="4" t="n"/>
+      <c r="I124" s="4" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="8" t="inlineStr">
+      <c r="A125" s="4" t="inlineStr">
         <is>
           <t>TC-1115</t>
         </is>
       </c>
-      <c r="B125" s="8" t="inlineStr">
+      <c r="B125" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C125" s="8" t="inlineStr">
+      <c r="C125" s="4" t="inlineStr">
         <is>
           <t>Auth after setup — test-connection</t>
         </is>
       </c>
-      <c r="D125" s="8" t="inlineStr">
+      <c r="D125" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/test-connection without token (after admin exists)</t>
         </is>
       </c>
-      <c r="E125" s="8" t="inlineStr">
+      <c r="E125" s="4" t="inlineStr">
         <is>
           <t>401</t>
         </is>
       </c>
-      <c r="F125" s="8" t="n"/>
-      <c r="G125" s="8" t="n"/>
-      <c r="H125" s="8" t="n"/>
-      <c r="I125" s="8" t="n"/>
+      <c r="F125" s="4" t="n"/>
+      <c r="G125" s="4" t="n"/>
+      <c r="H125" s="4" t="n"/>
+      <c r="I125" s="4" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="8" t="inlineStr">
+      <c r="A126" s="4" t="inlineStr">
         <is>
           <t>TC-1116</t>
         </is>
       </c>
-      <c r="B126" s="8" t="inlineStr">
+      <c r="B126" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C126" s="8" t="inlineStr">
+      <c r="C126" s="4" t="inlineStr">
         <is>
           <t>Auth after setup — provision</t>
         </is>
       </c>
-      <c r="D126" s="8" t="inlineStr">
+      <c r="D126" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/provision without token (after admin exists)</t>
         </is>
       </c>
-      <c r="E126" s="8" t="inlineStr">
+      <c r="E126" s="4" t="inlineStr">
         <is>
           <t>401</t>
         </is>
       </c>
-      <c r="F126" s="8" t="n"/>
-      <c r="G126" s="8" t="n"/>
-      <c r="H126" s="8" t="n"/>
-      <c r="I126" s="8" t="n"/>
+      <c r="F126" s="4" t="n"/>
+      <c r="G126" s="4" t="n"/>
+      <c r="H126" s="4" t="n"/>
+      <c r="I126" s="4" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="8" t="inlineStr">
+      <c r="A127" s="4" t="inlineStr">
         <is>
           <t>TC-1117</t>
         </is>
       </c>
-      <c r="B127" s="8" t="inlineStr">
+      <c r="B127" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C127" s="8" t="inlineStr">
+      <c r="C127" s="4" t="inlineStr">
         <is>
           <t>Password redaction</t>
         </is>
       </c>
-      <c r="D127" s="8" t="inlineStr">
+      <c r="D127" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/provision and check response</t>
         </is>
       </c>
-      <c r="E127" s="8" t="inlineStr">
+      <c r="E127" s="4" t="inlineStr">
         <is>
           <t>No password in response body</t>
         </is>
       </c>
-      <c r="F127" s="8" t="n"/>
-      <c r="G127" s="8" t="n"/>
-      <c r="H127" s="8" t="n"/>
-      <c r="I127" s="8" t="n"/>
+      <c r="F127" s="4" t="n"/>
+      <c r="G127" s="4" t="n"/>
+      <c r="H127" s="4" t="n"/>
+      <c r="I127" s="4" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="8" t="inlineStr">
+      <c r="A128" s="4" t="inlineStr">
         <is>
           <t>TC-1118</t>
         </is>
       </c>
-      <c r="B128" s="8" t="inlineStr">
+      <c r="B128" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C128" s="8" t="inlineStr">
+      <c r="C128" s="4" t="inlineStr">
         <is>
           <t>Re-provision blocked</t>
         </is>
       </c>
-      <c r="D128" s="8" t="inlineStr">
+      <c r="D128" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/provision after successful provisioning (no force)</t>
         </is>
       </c>
-      <c r="E128" s="8" t="inlineStr">
+      <c r="E128" s="4" t="inlineStr">
         <is>
           <t>409, already provisioned</t>
         </is>
       </c>
-      <c r="F128" s="8" t="n"/>
-      <c r="G128" s="8" t="n"/>
-      <c r="H128" s="8" t="n"/>
-      <c r="I128" s="8" t="n"/>
+      <c r="F128" s="4" t="n"/>
+      <c r="G128" s="4" t="n"/>
+      <c r="H128" s="4" t="n"/>
+      <c r="I128" s="4" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="8" t="inlineStr">
+      <c r="A129" s="4" t="inlineStr">
         <is>
           <t>TC-1119</t>
         </is>
       </c>
-      <c r="B129" s="8" t="inlineStr">
+      <c r="B129" s="4" t="inlineStr">
         <is>
           <t>12.11 Database Provisioning</t>
         </is>
       </c>
-      <c r="C129" s="8" t="inlineStr">
+      <c r="C129" s="4" t="inlineStr">
         <is>
           <t>Force re-provision</t>
         </is>
       </c>
-      <c r="D129" s="8" t="inlineStr">
+      <c r="D129" s="4" t="inlineStr">
         <is>
           <t>POST /setup/database/provision with "force": true after successful provisioning</t>
         </is>
       </c>
-      <c r="E129" s="8" t="inlineStr">
+      <c r="E129" s="4" t="inlineStr">
         <is>
           <t>200, returns database, user, migrations_applied</t>
         </is>
       </c>
-      <c r="F129" s="8" t="n"/>
-      <c r="G129" s="8" t="n"/>
-      <c r="H129" s="8" t="n"/>
-      <c r="I129" s="8" t="n"/>
+      <c r="F129" s="4" t="n"/>
+      <c r="G129" s="4" t="n"/>
+      <c r="H129" s="4" t="n"/>
+      <c r="I129" s="4" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="4" t="inlineStr">
+        <is>
+          <t>TC-1120</t>
+        </is>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — DB unreachable, no JWT</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="inlineStr">
+        <is>
+          <t>503, database unavailable message</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="n"/>
+      <c r="G130" s="4" t="n"/>
+      <c r="H130" s="4" t="n"/>
+      <c r="I130" s="4" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="8" t="inlineStr">
+      <c r="A131" s="4" t="inlineStr">
+        <is>
+          <t>TC-1121</t>
+        </is>
+      </c>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C131" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — DB unreachable, admin JWT</t>
+        </is>
+      </c>
+      <c r="D131" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+        </is>
+      </c>
+      <c r="E131" s="4" t="inlineStr">
+        <is>
+          <t>Request proceeds (not blocked by 503)</t>
+        </is>
+      </c>
+      <c r="F131" s="4" t="n"/>
+      <c r="G131" s="4" t="n"/>
+      <c r="H131" s="4" t="n"/>
+      <c r="I131" s="4" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B131" s="8" t="n">
-        <v>114</v>
-      </c>
-      <c r="C131" s="8" t="n"/>
-      <c r="D131" s="8" t="n"/>
-      <c r="E131" s="8" t="n"/>
-      <c r="F131" s="8" t="n"/>
-      <c r="G131" s="8" t="n"/>
-      <c r="H131" s="8" t="n"/>
-      <c r="I131" s="8" t="n"/>
+      <c r="B133" s="5" t="n">
+        <v>119</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Enforce admin authentication for force re-provisioning in database setup endpoints
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I133"/>
+  <dimension ref="A1:I134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4272,12 +4272,12 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>Force re-provision</t>
+          <t>Force re-provision (admin)</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>POST /setup/database/provision with "force": true after successful provisioning</t>
+          <t>POST /setup/database/provision with "force": true and admin token after successful provisioning</t>
         </is>
       </c>
       <c r="E129" s="4" t="inlineStr">
@@ -4303,17 +4303,17 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, no JWT</t>
+          <t>Force rejected unauthenticated</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
+          <t>POST /setup/database/provision with "force": true during initial setup (no admin exists)</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>503, database unavailable message</t>
+          <t>403, force requires admin</t>
         </is>
       </c>
       <c r="F130" s="4" t="n"/>
@@ -4334,17 +4334,17 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>Fail-closed — DB unreachable, admin JWT</t>
+          <t>Fail-closed — DB unreachable, no JWT</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection without token</t>
         </is>
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>Request proceeds (not blocked by 503)</t>
+          <t>503, database unavailable message</t>
         </is>
       </c>
       <c r="F131" s="4" t="n"/>
@@ -4352,14 +4352,45 @@
       <c r="H131" s="4" t="n"/>
       <c r="I131" s="4" t="n"/>
     </row>
-    <row r="133">
-      <c r="A133" s="5" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>TC-1122</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — DB unreachable, admin JWT</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/test-connection with valid admin token</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="inlineStr">
+        <is>
+          <t>Request proceeds (not blocked by 503)</t>
+        </is>
+      </c>
+      <c r="F132" s="4" t="n"/>
+      <c r="G132" s="4" t="n"/>
+      <c r="H132" s="4" t="n"/>
+      <c r="I132" s="4" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B133" s="5" t="n">
-        <v>119</v>
+      <c r="B134" s="5" t="n">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add DatabaseStatusUnknownError exception and update provisioning logic to handle transient database connectivity issues
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I134"/>
+  <dimension ref="A1:I136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4383,14 +4383,76 @@
       <c r="H132" s="4" t="n"/>
       <c r="I132" s="4" t="n"/>
     </row>
+    <row r="133">
+      <c r="A133" s="4" t="inlineStr">
+        <is>
+          <t>TC-1123</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — provision state unknown</t>
+        </is>
+      </c>
+      <c r="D133" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/provision without "force": true</t>
+        </is>
+      </c>
+      <c r="E133" s="4" t="inlineStr">
+        <is>
+          <t>503, cannot determine provisioning state</t>
+        </is>
+      </c>
+      <c r="F133" s="4" t="n"/>
+      <c r="G133" s="4" t="n"/>
+      <c r="H133" s="4" t="n"/>
+      <c r="I133" s="4" t="n"/>
+    </row>
     <row r="134">
-      <c r="A134" s="5" t="inlineStr">
+      <c r="A134" s="4" t="inlineStr">
+        <is>
+          <t>TC-1124</t>
+        </is>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="inlineStr">
+        <is>
+          <t>Force bypasses state check</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>Stop PostgreSQL, POST /setup/database/provision with "force": true and admin token</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="inlineStr">
+        <is>
+          <t>Proceeds to provisioning (no 503 from state check)</t>
+        </is>
+      </c>
+      <c r="F134" s="4" t="n"/>
+      <c r="G134" s="4" t="n"/>
+      <c r="H134" s="4" t="n"/>
+      <c r="I134" s="4" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B134" s="5" t="n">
-        <v>120</v>
+      <c r="B136" s="5" t="n">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance database provisioning logic to treat reachable but unmigrated databases as initial setup, and update tests accordingly
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I136"/>
+  <dimension ref="A1:I137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4445,14 +4445,45 @@
       <c r="H134" s="4" t="n"/>
       <c r="I134" s="4" t="n"/>
     </row>
-    <row r="136">
-      <c r="A136" s="5" t="inlineStr">
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>TC-1125</t>
+        </is>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>Unmigrated DB treated as initial setup</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>Drop user_roles table (or use a fresh empty database), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>200, request allowed (not 503)</t>
+        </is>
+      </c>
+      <c r="F135" s="4" t="n"/>
+      <c r="G135" s="4" t="n"/>
+      <c r="H135" s="4" t="n"/>
+      <c r="I135" s="4" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B136" s="5" t="n">
-        <v>122</v>
+      <c r="B137" s="5" t="n">
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance database provisioning logic to treat missing databases and roles as unprovisioned, allowing initial setup to proceed without force. Update tests to verify behavior for various provisioning states.
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I137"/>
+  <dimension ref="A1:I138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4476,14 +4476,45 @@
       <c r="H135" s="4" t="n"/>
       <c r="I135" s="4" t="n"/>
     </row>
-    <row r="137">
-      <c r="A137" s="5" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="4" t="inlineStr">
+        <is>
+          <t>TC-1126</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>Fresh install — DB/role missing</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>With PostgreSQL running but the application database or role not yet created, POST /setup/database/provision without force</t>
+        </is>
+      </c>
+      <c r="E136" s="4" t="inlineStr">
+        <is>
+          <t>200, provisioning proceeds (not 503)</t>
+        </is>
+      </c>
+      <c r="F136" s="4" t="n"/>
+      <c r="G136" s="4" t="n"/>
+      <c r="H136" s="4" t="n"/>
+      <c r="I136" s="4" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B137" s="5" t="n">
-        <v>123</v>
+      <c r="B138" s="5" t="n">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance fail-closed behavior for database provisioning by distinguishing between operational errors and initial setup conditions. Update tests to verify that operational errors and unexpected exceptions do not trigger initial setup, ensuring proper authentication requirements are enforced.
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I138"/>
+  <dimension ref="A1:I140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4507,14 +4507,76 @@
       <c r="H136" s="4" t="n"/>
       <c r="I136" s="4" t="n"/>
     </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>TC-1127</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — OperationalError on reachable DB</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>Revoke SELECT on user_roles (or simulate permission denied), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="inlineStr">
+        <is>
+          <t>503, does NOT grant unauthenticated access</t>
+        </is>
+      </c>
+      <c r="F137" s="4" t="n"/>
+      <c r="G137" s="4" t="n"/>
+      <c r="H137" s="4" t="n"/>
+      <c r="I137" s="4" t="n"/>
+    </row>
     <row r="138">
-      <c r="A138" s="5" t="inlineStr">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>TC-1128</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>Fail-closed — unexpected error</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>Trigger an unexpected exception from admin-check (e.g. coding bug), POST /setup/database/test-connection without token</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="inlineStr">
+        <is>
+          <t>503, does NOT grant unauthenticated access</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="n"/>
+      <c r="G138" s="4" t="n"/>
+      <c r="H138" s="4" t="n"/>
+      <c r="I138" s="4" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B138" s="5" t="n">
-        <v>124</v>
+      <c r="B140" s="5" t="n">
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance database provisioning logic to ensure that migrations must succeed before writing to .env and reinitializing the engine. Update tests to verify behavior for migration failures and .env write issues.
</commit_message>
<xml_diff>
--- a/documents/operations/ecube-qa-test-cases.xlsx
+++ b/documents/operations/ecube-qa-test-cases.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I140"/>
+  <dimension ref="A1:I143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4569,14 +4569,107 @@
       <c r="H138" s="4" t="n"/>
       <c r="I138" s="4" t="n"/>
     </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>TC-1129</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>Provision — migration failure</t>
+        </is>
+      </c>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision with valid credentials but a broken Alembic migration (e.g. conflicting schema)</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="inlineStr">
+        <is>
+          <t>500, "migration failed" message; .env not updated, engine not swapped</t>
+        </is>
+      </c>
+      <c r="F139" s="4" t="n"/>
+      <c r="G139" s="4" t="n"/>
+      <c r="H139" s="4" t="n"/>
+      <c r="I139" s="4" t="n"/>
+    </row>
     <row r="140">
-      <c r="A140" s="5" t="inlineStr">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>TC-1130</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>Provision — .env write failure</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision after making .env read-only (or disk full)</t>
+        </is>
+      </c>
+      <c r="E140" s="4" t="inlineStr">
+        <is>
+          <t>500, "failed to persist" message; engine not swapped</t>
+        </is>
+      </c>
+      <c r="F140" s="4" t="n"/>
+      <c r="G140" s="4" t="n"/>
+      <c r="H140" s="4" t="n"/>
+      <c r="I140" s="4" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="4" t="inlineStr">
+        <is>
+          <t>TC-1131</t>
+        </is>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t>12.11 Database Provisioning</t>
+        </is>
+      </c>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>Provision — engine reinit failure</t>
+        </is>
+      </c>
+      <c r="D141" s="4" t="inlineStr">
+        <is>
+          <t>POST /setup/database/provision while another reinit is in progress (lock contention)</t>
+        </is>
+      </c>
+      <c r="E141" s="4" t="inlineStr">
+        <is>
+          <t>500, "engine could not be switched" message; .env already written</t>
+        </is>
+      </c>
+      <c r="F141" s="4" t="n"/>
+      <c r="G141" s="4" t="n"/>
+      <c r="H141" s="4" t="n"/>
+      <c r="I141" s="4" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
         <is>
           <t>Total Test Cases:</t>
         </is>
       </c>
-      <c r="B140" s="5" t="n">
-        <v>126</v>
+      <c r="B143" s="5" t="n">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>